<commit_message>
update: sku master file
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804C7222-F2CC-4777-8B44-59C7D18A6658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF45B70-8626-4E22-B6DB-5BA58E9F8F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$481</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$480</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3167" uniqueCount="1649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3166" uniqueCount="1649">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -5651,7 +5651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:I481"/>
+  <dimension ref="A1:I480"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -18234,11 +18234,6 @@
       <c r="H480" s="13"/>
       <c r="I480" s="15">
         <v>0</v>
-      </c>
-    </row>
-    <row r="481" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A481" s="1" t="s">
-        <v>1220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: skip temp Excel lock files in AMS step3
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,18 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2FCAE9-BF71-440F-B5BB-516CA2AC2303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B565C51F-9CF5-40E7-A9EB-92BD02335C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$839</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$833</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4978" uniqueCount="2709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4938" uniqueCount="2708">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -8143,9 +8140,6 @@
   </si>
   <si>
     <t>B0GN8RQJRG</t>
-  </si>
-  <si>
-    <t>Electronic Keyboard</t>
   </si>
   <si>
     <t>B0GKNGWLJ2</t>
@@ -8173,7 +8167,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8216,13 +8210,6 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -8284,7 +8271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -8333,9 +8320,6 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8523,2542 +8507,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Main"/>
-      <sheetName val="Margin Structure"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="B1" t="str">
-            <v>SKU</v>
-          </cell>
-          <cell r="C1" t="str">
-            <v>ASIN</v>
-          </cell>
-          <cell r="E1" t="str">
-            <v>Model</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="B2" t="str">
-            <v>FBA75673</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>B0B4DPX2J2</v>
-          </cell>
-          <cell r="E2" t="str">
-            <v>AM-C1</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="B3" t="str">
-            <v>FBA76864</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>B0BPLZ5CGV</v>
-          </cell>
-          <cell r="E3" t="str">
-            <v>AI-04 Red</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="B4" t="str">
-            <v>FBA79005</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>B0CKHVHVQ1</v>
-          </cell>
-          <cell r="E4" t="str">
-            <v>AM-W45</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="B5" t="str">
-            <v>FBA79380</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>B0D3M1B4Z8</v>
-          </cell>
-          <cell r="E5" t="str">
-            <v>AM-C46</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="B6" t="str">
-            <v>FBA75692</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>B0B4G1HPL5</v>
-          </cell>
-          <cell r="E6" t="str">
-            <v>AM-C11</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="B7" t="str">
-            <v>FBA75691</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>B0B4G5JG4P</v>
-          </cell>
-          <cell r="E7" t="str">
-            <v>AM-W14</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="B8" t="str">
-            <v>FBA79107</v>
-          </cell>
-          <cell r="C8" t="str">
-            <v>B0CM9P5CCK</v>
-          </cell>
-          <cell r="E8" t="str">
-            <v>AM-W17</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="B9" t="str">
-            <v>FBA75674</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>B0B4G19R58</v>
-          </cell>
-          <cell r="E9" t="str">
-            <v>AM-C2</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="B10" t="str">
-            <v>FBA79109</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>B0CM9HYVDM</v>
-          </cell>
-          <cell r="E10" t="str">
-            <v>AM-W18</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="B11" t="str">
-            <v>FBA75675</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>B0B4G8ZB64</v>
-          </cell>
-          <cell r="E11" t="str">
-            <v>AM-C3</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12" t="str">
-            <v>FBA79070</v>
-          </cell>
-          <cell r="C12" t="str">
-            <v>B0CLH7G5WH</v>
-          </cell>
-          <cell r="E12" t="str">
-            <v>AI-02 2x2| Metallic Red</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="B13" t="str">
-            <v>FBA79103</v>
-          </cell>
-          <cell r="C13" t="str">
-            <v>B0CM6NTWBP</v>
-          </cell>
-          <cell r="E13" t="str">
-            <v>AI-10</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="B14" t="str">
-            <v>FBA75690</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>B0B4K87PR4</v>
-          </cell>
-          <cell r="E14" t="str">
-            <v>AM-C10</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="B15" t="str">
-            <v>FBA78975</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>B0CF5TCQKL</v>
-          </cell>
-          <cell r="E15" t="str">
-            <v>AA-21</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="B16" t="str">
-            <v>FBA78973</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v>B0CF5R3V95</v>
-          </cell>
-          <cell r="E16" t="str">
-            <v>AA-19</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="B17" t="str">
-            <v>FBA76414</v>
-          </cell>
-          <cell r="C17" t="str">
-            <v>B0BLJVJ2GN</v>
-          </cell>
-          <cell r="E17" t="str">
-            <v>AA-05</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="B18" t="str">
-            <v>FBA79379</v>
-          </cell>
-          <cell r="C18" t="str">
-            <v>B0D3LZWTHV</v>
-          </cell>
-          <cell r="E18" t="str">
-            <v>AM-C45</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="B19" t="str">
-            <v>FBA78925</v>
-          </cell>
-          <cell r="C19" t="str">
-            <v>B0CBC7QMNV</v>
-          </cell>
-          <cell r="E19" t="str">
-            <v>AM-C11X</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="B20" t="str">
-            <v>FBA75688</v>
-          </cell>
-          <cell r="C20" t="str">
-            <v>B0B4G763WS</v>
-          </cell>
-          <cell r="E20" t="str">
-            <v>AM-W12</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="B21" t="str">
-            <v>FBA76744</v>
-          </cell>
-          <cell r="C21" t="str">
-            <v>B0BLK7VQ2N</v>
-          </cell>
-          <cell r="E21" t="str">
-            <v xml:space="preserve">AM-K3 </v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="B22" t="str">
-            <v>FBA78974</v>
-          </cell>
-          <cell r="C22" t="str">
-            <v>B0CF5RRTDJ</v>
-          </cell>
-          <cell r="E22" t="str">
-            <v>AA-20</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="B23" t="str">
-            <v>FBA79447</v>
-          </cell>
-          <cell r="C23" t="str">
-            <v>B0DFMLXD9S</v>
-          </cell>
-          <cell r="E23" t="str">
-            <v>AM-W34</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="B24" t="str">
-            <v>FBA75686</v>
-          </cell>
-          <cell r="C24" t="str">
-            <v>B0B4G89VQJ</v>
-          </cell>
-          <cell r="E24" t="str">
-            <v>AM-W10</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="B25" t="str">
-            <v>FBA79011</v>
-          </cell>
-          <cell r="C25" t="str">
-            <v>B0CH4RNWJX</v>
-          </cell>
-          <cell r="E25" t="str">
-            <v>AM-C43</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="B26" t="str">
-            <v>FBA79064</v>
-          </cell>
-          <cell r="C26" t="str">
-            <v>B0CJR76Y7G</v>
-          </cell>
-          <cell r="E26" t="str">
-            <v>AA-25</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="B27" t="str">
-            <v>FBA75679</v>
-          </cell>
-          <cell r="C27" t="str">
-            <v>B0B4JRQP22</v>
-          </cell>
-          <cell r="E27" t="str">
-            <v>AA-02</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="B28" t="str">
-            <v>FBA79449</v>
-          </cell>
-          <cell r="C28" t="str">
-            <v>B0DFMNGFTD</v>
-          </cell>
-          <cell r="E28" t="str">
-            <v>AM-W36</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="B29" t="str">
-            <v>FBA79106</v>
-          </cell>
-          <cell r="C29" t="str">
-            <v>B0CM9KJZWQ</v>
-          </cell>
-          <cell r="E29" t="str">
-            <v>AM-C44</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="B30" t="str">
-            <v>FBA76742</v>
-          </cell>
-          <cell r="C30" t="str">
-            <v>B0BLKBJ5HN</v>
-          </cell>
-          <cell r="E30" t="str">
-            <v xml:space="preserve">AM-K1 </v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="B31" t="str">
-            <v>FBA79355</v>
-          </cell>
-          <cell r="C31" t="str">
-            <v>B0D3M86SH1</v>
-          </cell>
-          <cell r="E31" t="str">
-            <v>AA-19BL</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="B32" t="str">
-            <v>FBA76863</v>
-          </cell>
-          <cell r="C32" t="str">
-            <v>B0BPM2T7BQ</v>
-          </cell>
-          <cell r="E32" t="str">
-            <v xml:space="preserve">AI-03	</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="B33" t="str">
-            <v>FBA75677</v>
-          </cell>
-          <cell r="C33" t="str">
-            <v>B0B4KC7VBM</v>
-          </cell>
-          <cell r="E33" t="str">
-            <v>AM-C5</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="B34" t="str">
-            <v>FBA77171</v>
-          </cell>
-          <cell r="C34" t="str">
-            <v>B0CH4VCD6R</v>
-          </cell>
-          <cell r="E34" t="str">
-            <v>AC-6XL</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="B35" t="str">
-            <v>FBA79105</v>
-          </cell>
-          <cell r="C35" t="str">
-            <v>B0CM6WH4ZT</v>
-          </cell>
-          <cell r="E35" t="str">
-            <v>AI-12</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="B36" t="str">
-            <v>FBA79230</v>
-          </cell>
-          <cell r="C36" t="str">
-            <v>B0CX1XK5R6</v>
-          </cell>
-          <cell r="E36" t="str">
-            <v>AM-W46</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="B37" t="str">
-            <v>FBA78960</v>
-          </cell>
-          <cell r="C37" t="str">
-            <v>B0CBCB82MT</v>
-          </cell>
-          <cell r="E37" t="str">
-            <v>AM-C39</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="B38" t="str">
-            <v>FBA75684</v>
-          </cell>
-          <cell r="C38" t="str">
-            <v>B0B4G7VWXD</v>
-          </cell>
-          <cell r="E38" t="str">
-            <v>AA-04</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="B39" t="str">
-            <v>FBA76723</v>
-          </cell>
-          <cell r="C39" t="str">
-            <v>B0BLKF46QG</v>
-          </cell>
-          <cell r="E39" t="str">
-            <v xml:space="preserve">AM-C20 </v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="B40" t="str">
-            <v>FBA76721</v>
-          </cell>
-          <cell r="C40" t="str">
-            <v>B0BLKB55BM</v>
-          </cell>
-          <cell r="E40" t="str">
-            <v xml:space="preserve">AM-C18 </v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="B41" t="str">
-            <v>FBA75681</v>
-          </cell>
-          <cell r="C41" t="str">
-            <v>B0B4FZS38V</v>
-          </cell>
-          <cell r="E41" t="str">
-            <v>AM-C7</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="B42" t="str">
-            <v>FBA75678</v>
-          </cell>
-          <cell r="C42" t="str">
-            <v>B0B4G8PH2P</v>
-          </cell>
-          <cell r="E42" t="str">
-            <v>AA-01</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="B43" t="str">
-            <v>FBA79446</v>
-          </cell>
-          <cell r="C43" t="str">
-            <v>B0DFMMTWLY</v>
-          </cell>
-          <cell r="E43" t="str">
-            <v>AM-W33</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="B44" t="str">
-            <v>FBA76862</v>
-          </cell>
-          <cell r="C44" t="str">
-            <v>B0BPLWW72Y</v>
-          </cell>
-          <cell r="E44" t="str">
-            <v>AM-C28</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="B45" t="str">
-            <v>FBA79010</v>
-          </cell>
-          <cell r="C45" t="str">
-            <v>B0CH4T2BJD</v>
-          </cell>
-          <cell r="E45" t="str">
-            <v>AM-C42</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="B46" t="str">
-            <v>FBA79104</v>
-          </cell>
-          <cell r="C46" t="str">
-            <v>B0CM6NVLT9</v>
-          </cell>
-          <cell r="E46" t="str">
-            <v>AI-11</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="B47" t="str">
-            <v>FBA76730</v>
-          </cell>
-          <cell r="C47" t="str">
-            <v>B0BLKB6FRR</v>
-          </cell>
-          <cell r="E47" t="str">
-            <v xml:space="preserve">AM-C27 </v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="B48" t="str">
-            <v>FBA76597</v>
-          </cell>
-          <cell r="C48" t="str">
-            <v>B0BQ7H7418</v>
-          </cell>
-          <cell r="E48" t="str">
-            <v>AA-06</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="B49" t="str">
-            <v>FBA79465</v>
-          </cell>
-          <cell r="C49" t="str">
-            <v>B0DFMQCGT1</v>
-          </cell>
-          <cell r="E49" t="str">
-            <v>AM-W21</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="B50" t="str">
-            <v>FBA79445</v>
-          </cell>
-          <cell r="C50" t="str">
-            <v>B0DFMLS8JG</v>
-          </cell>
-          <cell r="E50" t="str">
-            <v>AM-W32</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="B51" t="str">
-            <v>FBA75676</v>
-          </cell>
-          <cell r="C51" t="str">
-            <v>B0B4DS678Q</v>
-          </cell>
-          <cell r="E51" t="str">
-            <v>AM-C4</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="B52" t="str">
-            <v>FBA78986</v>
-          </cell>
-          <cell r="C52" t="str">
-            <v>B0CF5WXWFH</v>
-          </cell>
-          <cell r="E52" t="str">
-            <v>AB-01</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="B53" t="str">
-            <v>FBA75689</v>
-          </cell>
-          <cell r="C53" t="str">
-            <v>B0B4G59Y8W</v>
-          </cell>
-          <cell r="E53" t="str">
-            <v>AM-W13</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="B54" t="str">
-            <v>FBA75680</v>
-          </cell>
-          <cell r="C54" t="str">
-            <v>B0B4G1PXWV</v>
-          </cell>
-          <cell r="E54" t="str">
-            <v>AM-C6</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="B55" t="str">
-            <v>FBA78205</v>
-          </cell>
-          <cell r="C55" t="str">
-            <v>B0C539RBGL</v>
-          </cell>
-          <cell r="E55" t="str">
-            <v>AM-C32</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="B56" t="str">
-            <v>FBA76729</v>
-          </cell>
-          <cell r="C56" t="str">
-            <v>B0BLNDQ757</v>
-          </cell>
-          <cell r="E56" t="str">
-            <v xml:space="preserve">AM-C26 </v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="B57" t="str">
-            <v>FBA78976</v>
-          </cell>
-          <cell r="C57" t="str">
-            <v>B0CF5SHL15</v>
-          </cell>
-          <cell r="E57" t="str">
-            <v>AA-22</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="B58" t="str">
-            <v>FBA76735</v>
-          </cell>
-          <cell r="C58" t="str">
-            <v>B0BLKGPL4X</v>
-          </cell>
-          <cell r="E58" t="str">
-            <v xml:space="preserve">AA-08 </v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="B59" t="str">
-            <v>FBA79444</v>
-          </cell>
-          <cell r="C59" t="str">
-            <v>B0DFMLQBMC</v>
-          </cell>
-          <cell r="E59" t="str">
-            <v>AM-W20</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="B60" t="str">
-            <v>FBA76727</v>
-          </cell>
-          <cell r="C60" t="str">
-            <v>B0BLKCDRNB</v>
-          </cell>
-          <cell r="E60" t="str">
-            <v xml:space="preserve">AM-C24 </v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="B61" t="str">
-            <v>FBA75683</v>
-          </cell>
-          <cell r="C61" t="str">
-            <v>B0B4G94VP3</v>
-          </cell>
-          <cell r="E61" t="str">
-            <v>AA-03</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="B62" t="str">
-            <v>FBA79016</v>
-          </cell>
-          <cell r="C62" t="str">
-            <v>B0CH4R1V6S</v>
-          </cell>
-          <cell r="E62" t="str">
-            <v>AM-C3a</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="B63" t="str">
-            <v>FBA75687</v>
-          </cell>
-          <cell r="C63" t="str">
-            <v>B0B4G5ZLTB</v>
-          </cell>
-          <cell r="E63" t="str">
-            <v>AM-W11</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="B64" t="str">
-            <v>FBA78203</v>
-          </cell>
-          <cell r="C64" t="str">
-            <v>B0C4YTNJG7</v>
-          </cell>
-          <cell r="E64" t="str">
-            <v>AM-C30</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="B65" t="str">
-            <v>FBA79009</v>
-          </cell>
-          <cell r="C65" t="str">
-            <v>B0CH4PMR8K</v>
-          </cell>
-          <cell r="E65" t="str">
-            <v>AM-C41</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="B66" t="str">
-            <v>FBA79108</v>
-          </cell>
-          <cell r="C66" t="str">
-            <v>B0CM9L1QZG</v>
-          </cell>
-          <cell r="E66" t="str">
-            <v>AM-W16</v>
-          </cell>
-        </row>
-        <row r="67">
-          <cell r="B67" t="str">
-            <v>FBA79008</v>
-          </cell>
-          <cell r="C67" t="str">
-            <v>B0CH4RT4P8</v>
-          </cell>
-          <cell r="E67" t="str">
-            <v>AI-06</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="B68" t="str">
-            <v>FBA79448</v>
-          </cell>
-          <cell r="C68" t="str">
-            <v>B0DFMKY4TT</v>
-          </cell>
-          <cell r="E68" t="str">
-            <v>AM-W35</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="B69" t="str">
-            <v>FBA78961</v>
-          </cell>
-          <cell r="C69" t="str">
-            <v>B0CBCB9S14</v>
-          </cell>
-          <cell r="E69" t="str">
-            <v>AM-C40</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="B70" t="str">
-            <v>FBA78206</v>
-          </cell>
-          <cell r="C70" t="str">
-            <v>B0C4YSV3XL</v>
-          </cell>
-          <cell r="E70" t="str">
-            <v>AM-W15</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="B71" t="str">
-            <v>FBA79356</v>
-          </cell>
-          <cell r="C71" t="str">
-            <v>B0D3Q2T5XX</v>
-          </cell>
-          <cell r="E71" t="str">
-            <v>AA-19WL</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="B72" t="str">
-            <v>FBA78204</v>
-          </cell>
-          <cell r="C72" t="str">
-            <v>B0C4YT43Z3</v>
-          </cell>
-          <cell r="E72" t="str">
-            <v>AM-C31</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="B73" t="str">
-            <v>FBA76743</v>
-          </cell>
-          <cell r="C73" t="str">
-            <v>B0BLK8PXNY</v>
-          </cell>
-          <cell r="E73" t="str">
-            <v xml:space="preserve">AM-K2 </v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="B74" t="str">
-            <v>FBA76728</v>
-          </cell>
-          <cell r="C74" t="str">
-            <v>B0BLNCP74M</v>
-          </cell>
-          <cell r="E74" t="str">
-            <v xml:space="preserve">AM-C25 </v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="B75" t="str">
-            <v>FBA76716</v>
-          </cell>
-          <cell r="C75" t="str">
-            <v>B0BLK8DNPD</v>
-          </cell>
-          <cell r="E75" t="str">
-            <v xml:space="preserve">AM-C13 </v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="B76" t="str">
-            <v>FBA78423</v>
-          </cell>
-          <cell r="C76" t="str">
-            <v>B0C598Q6PT</v>
-          </cell>
-          <cell r="E76" t="str">
-            <v>AM-C36</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="B77" t="str">
-            <v>FBA78424</v>
-          </cell>
-          <cell r="C77" t="str">
-            <v>B0C55MY66L</v>
-          </cell>
-          <cell r="E77" t="str">
-            <v>AM-C37</v>
-          </cell>
-        </row>
-        <row r="78">
-          <cell r="B78" t="str">
-            <v>FBA78420</v>
-          </cell>
-          <cell r="C78" t="str">
-            <v>B0C5957W3P</v>
-          </cell>
-          <cell r="E78" t="str">
-            <v>AM-C33</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="B79" t="str">
-            <v>FBA77011</v>
-          </cell>
-          <cell r="C79" t="str">
-            <v>B0BPMN89NG</v>
-          </cell>
-          <cell r="E79" t="str">
-            <v>AM-C29</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="B80" t="str">
-            <v>FBA78425</v>
-          </cell>
-          <cell r="C80" t="str">
-            <v>B0C55QXL83</v>
-          </cell>
-          <cell r="E80" t="str">
-            <v>AM-C38</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="B81" t="str">
-            <v>FBA78972</v>
-          </cell>
-          <cell r="C81" t="str">
-            <v>B0CF5T89FT</v>
-          </cell>
-          <cell r="E81" t="str">
-            <v>AA-18</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="B82" t="str">
-            <v>FBA79014</v>
-          </cell>
-          <cell r="C82" t="str">
-            <v>B0CH4WFQF6</v>
-          </cell>
-          <cell r="E82" t="str">
-            <v>AI-09</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="B83" t="str">
-            <v>FBA75685</v>
-          </cell>
-          <cell r="C83" t="str">
-            <v>B0B4FXDHXW</v>
-          </cell>
-          <cell r="E83" t="str">
-            <v>AM-C9</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="B84" t="str">
-            <v>FBA76722</v>
-          </cell>
-          <cell r="C84" t="str">
-            <v>B0BLKDC4PP</v>
-          </cell>
-          <cell r="E84" t="str">
-            <v xml:space="preserve">AM-C19 </v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="B85" t="str">
-            <v>FBA76737</v>
-          </cell>
-          <cell r="C85" t="str">
-            <v>B0C59G1C4N</v>
-          </cell>
-          <cell r="E85" t="str">
-            <v>AA-10</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="B86" t="str">
-            <v>FBA76720</v>
-          </cell>
-          <cell r="C86" t="str">
-            <v>B0BLKCWZQD</v>
-          </cell>
-          <cell r="E86" t="str">
-            <v xml:space="preserve">AM-C17 </v>
-          </cell>
-        </row>
-        <row r="87">
-          <cell r="B87" t="str">
-            <v>FBA78419</v>
-          </cell>
-          <cell r="C87" t="str">
-            <v>B0C55M2GBN</v>
-          </cell>
-          <cell r="E87" t="str">
-            <v>AM-A1</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="B88" t="str">
-            <v>FBA78421</v>
-          </cell>
-          <cell r="C88" t="str">
-            <v>B0C594FZLM</v>
-          </cell>
-          <cell r="E88" t="str">
-            <v>AM-C34</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="B89" t="str">
-            <v>FBA78971</v>
-          </cell>
-          <cell r="C89" t="str">
-            <v>B0CF5TDLFH</v>
-          </cell>
-          <cell r="E89" t="str">
-            <v>AA-17</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="B90" t="str">
-            <v>FBA75682</v>
-          </cell>
-          <cell r="C90" t="str">
-            <v>B0B4FVV78V</v>
-          </cell>
-          <cell r="E90" t="str">
-            <v>AM-C8</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="B91" t="str">
-            <v>FBA76726</v>
-          </cell>
-          <cell r="C91" t="str">
-            <v>B0BLKD4815</v>
-          </cell>
-          <cell r="E91" t="str">
-            <v>AM-C23</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="B92" t="str">
-            <v>FBA76734</v>
-          </cell>
-          <cell r="C92" t="str">
-            <v>B0BLKHVCDX</v>
-          </cell>
-          <cell r="E92" t="str">
-            <v xml:space="preserve">AA-07 </v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="B93" t="str">
-            <v>FBA76739</v>
-          </cell>
-          <cell r="C93" t="str">
-            <v>B0BLRK37TB</v>
-          </cell>
-          <cell r="E93" t="str">
-            <v xml:space="preserve">AA-12 </v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="B94" t="str">
-            <v>FBA76732</v>
-          </cell>
-          <cell r="C94" t="str">
-            <v>B0BLKCB2JY</v>
-          </cell>
-          <cell r="E94" t="str">
-            <v>AI-01 / Q24</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="B95" t="str">
-            <v>FBA76717</v>
-          </cell>
-          <cell r="C95" t="str">
-            <v>B0BLK6P24G</v>
-          </cell>
-          <cell r="E95" t="str">
-            <v xml:space="preserve">AM-C14 </v>
-          </cell>
-        </row>
-        <row r="96">
-          <cell r="B96" t="str">
-            <v>FBA76718</v>
-          </cell>
-          <cell r="C96" t="str">
-            <v>B0BLKD8FVG</v>
-          </cell>
-          <cell r="E96" t="str">
-            <v xml:space="preserve">AM-C15 </v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="B97" t="str">
-            <v>FBA77010</v>
-          </cell>
-          <cell r="C97" t="str">
-            <v>B0BPMBMN3S</v>
-          </cell>
-          <cell r="E97" t="str">
-            <v>AI-04	Black</v>
-          </cell>
-        </row>
-        <row r="98">
-          <cell r="B98" t="str">
-            <v>FBA76715</v>
-          </cell>
-          <cell r="C98" t="str">
-            <v>B0BLK31PYH</v>
-          </cell>
-          <cell r="E98" t="str">
-            <v xml:space="preserve">AM-C12 </v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="B99" t="str">
-            <v>FBA78422</v>
-          </cell>
-          <cell r="C99" t="str">
-            <v>B0C598MNMC</v>
-          </cell>
-          <cell r="E99" t="str">
-            <v>AM-C35</v>
-          </cell>
-        </row>
-        <row r="100">
-          <cell r="B100" t="str">
-            <v>FBA76725</v>
-          </cell>
-          <cell r="C100" t="str">
-            <v>B0BLKCSJ7Z</v>
-          </cell>
-          <cell r="E100" t="str">
-            <v xml:space="preserve">AM-C22 </v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="B101" t="str">
-            <v>FBA79013</v>
-          </cell>
-          <cell r="C101" t="str">
-            <v>B0CH4TDGPG</v>
-          </cell>
-          <cell r="E101" t="str">
-            <v>AI-08</v>
-          </cell>
-        </row>
-        <row r="102">
-          <cell r="B102" t="str">
-            <v>FBA76738</v>
-          </cell>
-          <cell r="C102" t="str">
-            <v>B0BLRGCNRG</v>
-          </cell>
-          <cell r="E102" t="str">
-            <v xml:space="preserve">AA-11 </v>
-          </cell>
-        </row>
-        <row r="103">
-          <cell r="B103" t="str">
-            <v>FBAM75673</v>
-          </cell>
-          <cell r="C103" t="str">
-            <v>B0DFTVZPM8</v>
-          </cell>
-          <cell r="E103" t="str">
-            <v>AM-C1</v>
-          </cell>
-        </row>
-        <row r="104">
-          <cell r="B104" t="str">
-            <v>FBA76719</v>
-          </cell>
-          <cell r="C104" t="str">
-            <v>B0BLKCXQRT</v>
-          </cell>
-          <cell r="E104" t="str">
-            <v>AM-C16</v>
-          </cell>
-        </row>
-        <row r="105">
-          <cell r="B105" t="str">
-            <v>FBA76724</v>
-          </cell>
-          <cell r="C105" t="str">
-            <v>B0BLNC5D8L</v>
-          </cell>
-          <cell r="E105" t="str">
-            <v xml:space="preserve">AM-C21 </v>
-          </cell>
-        </row>
-        <row r="106">
-          <cell r="B106" t="str">
-            <v>FBA76733</v>
-          </cell>
-          <cell r="C106" t="str">
-            <v>B0BLKCJXZR</v>
-          </cell>
-          <cell r="E106" t="str">
-            <v>AI-02 / X2</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="B107" t="str">
-            <v>FBA76736</v>
-          </cell>
-          <cell r="C107" t="str">
-            <v>B0BLS63XCL</v>
-          </cell>
-          <cell r="E107" t="str">
-            <v xml:space="preserve">AA-09 </v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="B108" t="str">
-            <v>FBA76740</v>
-          </cell>
-          <cell r="C108" t="str">
-            <v>B0BLRKFBBP</v>
-          </cell>
-          <cell r="E108" t="str">
-            <v xml:space="preserve">AA-13 </v>
-          </cell>
-        </row>
-        <row r="109">
-          <cell r="B109" t="str">
-            <v>FBA76741</v>
-          </cell>
-          <cell r="C109" t="str">
-            <v>B0BLS2HJ68</v>
-          </cell>
-          <cell r="E109" t="str">
-            <v xml:space="preserve">AA-14 </v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="B110" t="str">
-            <v>FBA78207</v>
-          </cell>
-          <cell r="C110" t="str">
-            <v>B0C53CQV5Z</v>
-          </cell>
-          <cell r="E110" t="str">
-            <v>AA-15</v>
-          </cell>
-        </row>
-        <row r="111">
-          <cell r="B111" t="str">
-            <v>FBA79482</v>
-          </cell>
-          <cell r="C111" t="str">
-            <v>B0DXFPM4N2</v>
-          </cell>
-          <cell r="E111" t="str">
-            <v>AM-S1</v>
-          </cell>
-        </row>
-        <row r="112">
-          <cell r="B112" t="str">
-            <v>FBA78970</v>
-          </cell>
-          <cell r="C112" t="str">
-            <v>B0CF5T1LFR</v>
-          </cell>
-          <cell r="E112" t="str">
-            <v>AA-16</v>
-          </cell>
-        </row>
-        <row r="113">
-          <cell r="B113" t="str">
-            <v>FBA78977</v>
-          </cell>
-          <cell r="C113" t="str">
-            <v>B0CF5TVDRT</v>
-          </cell>
-          <cell r="E113" t="str">
-            <v>AA-23</v>
-          </cell>
-        </row>
-        <row r="114">
-          <cell r="B114" t="str">
-            <v>FBA78978</v>
-          </cell>
-          <cell r="C114" t="str">
-            <v>B0CF5PCL34</v>
-          </cell>
-          <cell r="E114" t="str">
-            <v>AA-24</v>
-          </cell>
-        </row>
-        <row r="115">
-          <cell r="B115" t="str">
-            <v>FBA79004</v>
-          </cell>
-          <cell r="C115" t="str">
-            <v>B0CF9BY345</v>
-          </cell>
-          <cell r="E115" t="str">
-            <v>AI-05</v>
-          </cell>
-        </row>
-        <row r="116">
-          <cell r="B116" t="str">
-            <v>FBA79012</v>
-          </cell>
-          <cell r="C116" t="str">
-            <v>B0CH4THGGM</v>
-          </cell>
-          <cell r="E116" t="str">
-            <v>AI-07</v>
-          </cell>
-        </row>
-        <row r="117">
-          <cell r="B117" t="str">
-            <v>FBA79389</v>
-          </cell>
-          <cell r="C117" t="str">
-            <v>B0D3M13T6H</v>
-          </cell>
-          <cell r="E117" t="str">
-            <v>AWB-01</v>
-          </cell>
-        </row>
-        <row r="118">
-          <cell r="B118" t="str">
-            <v>FBA77101</v>
-          </cell>
-          <cell r="C118" t="str">
-            <v>B07WLWN2ZT</v>
-          </cell>
-          <cell r="E118" t="str">
-            <v>TC-777</v>
-          </cell>
-        </row>
-        <row r="119">
-          <cell r="B119" t="str">
-            <v>FBA77104</v>
-          </cell>
-          <cell r="C119" t="str">
-            <v>B089SJGQBH</v>
-          </cell>
-          <cell r="E119" t="str">
-            <v>TC20</v>
-          </cell>
-        </row>
-        <row r="120">
-          <cell r="B120" t="str">
-            <v>FBA77111</v>
-          </cell>
-          <cell r="C120" t="str">
-            <v>B08CVP2HXP</v>
-          </cell>
-          <cell r="E120" t="str">
-            <v>TC30</v>
-          </cell>
-        </row>
-        <row r="121">
-          <cell r="B121" t="str">
-            <v>FBA79113</v>
-          </cell>
-          <cell r="C121" t="str">
-            <v>B0BTCXQQ6M</v>
-          </cell>
-          <cell r="E121" t="str">
-            <v>TC310</v>
-          </cell>
-        </row>
-        <row r="122">
-          <cell r="B122" t="str">
-            <v>FBA79114</v>
-          </cell>
-          <cell r="C122" t="str">
-            <v>B0CCV74CL7</v>
-          </cell>
-          <cell r="E122" t="str">
-            <v>TC310+</v>
-          </cell>
-        </row>
-        <row r="123">
-          <cell r="B123" t="str">
-            <v>FBA79116</v>
-          </cell>
-          <cell r="C123" t="str">
-            <v>B0BYHHSLPC</v>
-          </cell>
-          <cell r="E123" t="str">
-            <v>TC-777 PRO</v>
-          </cell>
-        </row>
-        <row r="124">
-          <cell r="B124" t="str">
-            <v>FBA77113</v>
-          </cell>
-          <cell r="C124" t="str">
-            <v>B01ISNU3X4</v>
-          </cell>
-          <cell r="E124" t="str">
-            <v>K1</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="B125" t="str">
-            <v>FBA79111</v>
-          </cell>
-          <cell r="C125" t="str">
-            <v>B0BRKFP94K</v>
-          </cell>
-          <cell r="E125" t="str">
-            <v>TD510</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="B126" t="str">
-            <v>FBA77110</v>
-          </cell>
-          <cell r="C126" t="str">
-            <v>B08NDB5NWP</v>
-          </cell>
-          <cell r="E126" t="str">
-            <v>TM20</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="B127" t="str">
-            <v>FBK77102</v>
-          </cell>
-          <cell r="C127" t="str">
-            <v>B07GVGMW59</v>
-          </cell>
-          <cell r="E127" t="str">
-            <v>G11</v>
-          </cell>
-        </row>
-        <row r="128">
-          <cell r="B128" t="str">
-            <v>FBA77117</v>
-          </cell>
-          <cell r="C128" t="str">
-            <v>B078WNW4YW</v>
-          </cell>
-          <cell r="E128" t="str">
-            <v>S20</v>
-          </cell>
-        </row>
-        <row r="129">
-          <cell r="B129" t="str">
-            <v>FBA79115</v>
-          </cell>
-          <cell r="C129" t="str">
-            <v>B0C8JDHLX9</v>
-          </cell>
-          <cell r="E129" t="str">
-            <v>T10</v>
-          </cell>
-        </row>
-        <row r="130">
-          <cell r="B130" t="str">
-            <v>FBA77106</v>
-          </cell>
-          <cell r="C130" t="str">
-            <v>B082W4B7SX</v>
-          </cell>
-          <cell r="E130" t="str">
-            <v>T20</v>
-          </cell>
-        </row>
-        <row r="131">
-          <cell r="B131" t="str">
-            <v>FBA77105</v>
-          </cell>
-          <cell r="C131" t="str">
-            <v>B089FVQD3Z</v>
-          </cell>
-          <cell r="E131" t="str">
-            <v>T30</v>
-          </cell>
-        </row>
-        <row r="132">
-          <cell r="B132" t="str">
-            <v>FBA79112</v>
-          </cell>
-          <cell r="C132" t="str">
-            <v>B0BRKDLXCD</v>
-          </cell>
-          <cell r="E132" t="str">
-            <v>T90</v>
-          </cell>
-        </row>
-        <row r="133">
-          <cell r="B133" t="str">
-            <v>FBA77103</v>
-          </cell>
-          <cell r="C133" t="str">
-            <v>B09Z5Q194D</v>
-          </cell>
-          <cell r="E133" t="str">
-            <v>ORCA001</v>
-          </cell>
-        </row>
-        <row r="134">
-          <cell r="B134" t="str">
-            <v>FBA77114</v>
-          </cell>
-          <cell r="C134" t="str">
-            <v>B07TSN2H9D</v>
-          </cell>
-          <cell r="E134" t="str">
-            <v>TC-2030</v>
-          </cell>
-        </row>
-        <row r="135">
-          <cell r="B135" t="str">
-            <v>FBA79574</v>
-          </cell>
-          <cell r="C135" t="str">
-            <v>B0B4WTHLX5</v>
-          </cell>
-          <cell r="E135" t="str">
-            <v>TC30S</v>
-          </cell>
-        </row>
-        <row r="136">
-          <cell r="B136" t="str">
-            <v>FBA79575</v>
-          </cell>
-          <cell r="C136" t="str">
-            <v>B0BG8CJXHH</v>
-          </cell>
-          <cell r="E136" t="str">
-            <v>TC30+</v>
-          </cell>
-        </row>
-        <row r="137">
-          <cell r="B137" t="str">
-            <v>FBA79576</v>
-          </cell>
-          <cell r="C137" t="str">
-            <v>B0BRCR2QQ7</v>
-          </cell>
-          <cell r="E137" t="str">
-            <v>TC30S+</v>
-          </cell>
-        </row>
-        <row r="138">
-          <cell r="B138" t="str">
-            <v>FBA79577</v>
-          </cell>
-          <cell r="C138" t="str">
-            <v>B0CSCT63BL</v>
-          </cell>
-          <cell r="E138" t="str">
-            <v>TM310</v>
-          </cell>
-        </row>
-        <row r="139">
-          <cell r="B139" t="str">
-            <v>FBA79578</v>
-          </cell>
-          <cell r="C139" t="str">
-            <v>B0CFKZ72N7</v>
-          </cell>
-          <cell r="E139" t="str">
-            <v>D5</v>
-          </cell>
-        </row>
-        <row r="140">
-          <cell r="B140" t="str">
-            <v>FBA79579</v>
-          </cell>
-          <cell r="C140" t="str">
-            <v>B0CQX4GVSB</v>
-          </cell>
-          <cell r="E140" t="str">
-            <v>D2</v>
-          </cell>
-        </row>
-        <row r="141">
-          <cell r="B141" t="str">
-            <v>FBA79582</v>
-          </cell>
-          <cell r="C141" t="str">
-            <v>B0CCVBQRFX</v>
-          </cell>
-          <cell r="E141" t="str">
-            <v>TD510+</v>
-          </cell>
-        </row>
-        <row r="142">
-          <cell r="B142" t="str">
-            <v>FBA79585</v>
-          </cell>
-          <cell r="C142" t="str">
-            <v>B0CFKHCQ8W</v>
-          </cell>
-          <cell r="E142" t="str">
-            <v>T20LP</v>
-          </cell>
-        </row>
-        <row r="143">
-          <cell r="B143" t="str">
-            <v>FBA79586</v>
-          </cell>
-          <cell r="C143" t="str">
-            <v>B0CH9JR3HL</v>
-          </cell>
-          <cell r="E143" t="str">
-            <v>TRL-20</v>
-          </cell>
-        </row>
-        <row r="144">
-          <cell r="B144" t="str">
-            <v>FBK79010</v>
-          </cell>
-          <cell r="C144" t="str">
-            <v>B0FLYJFC22</v>
-          </cell>
-          <cell r="E144" t="str">
-            <v>AM-C42 Duplicate</v>
-          </cell>
-        </row>
-        <row r="145">
-          <cell r="B145" t="str">
-            <v>FBA79722</v>
-          </cell>
-          <cell r="C145" t="str">
-            <v>B0F2HYY7JF</v>
-          </cell>
-          <cell r="E145" t="str">
-            <v>AM-W21 Duplicate</v>
-          </cell>
-        </row>
-        <row r="146">
-          <cell r="B146" t="str">
-            <v>FBA79909</v>
-          </cell>
-          <cell r="C146" t="str">
-            <v>B0FVM17Q4W</v>
-          </cell>
-          <cell r="E146" t="str">
-            <v>AM-W20 Duplicate</v>
-          </cell>
-        </row>
-        <row r="147">
-          <cell r="B147" t="str">
-            <v>FBK79009</v>
-          </cell>
-          <cell r="C147" t="str">
-            <v>B0FLYHJ6DK</v>
-          </cell>
-          <cell r="E147" t="str">
-            <v>AM-C41 Duplicate</v>
-          </cell>
-        </row>
-        <row r="148">
-          <cell r="B148" t="str">
-            <v>FBA79903</v>
-          </cell>
-          <cell r="C148" t="str">
-            <v>B0FR5DLXH9</v>
-          </cell>
-          <cell r="E148" t="str">
-            <v>AA-25M</v>
-          </cell>
-        </row>
-        <row r="149">
-          <cell r="B149" t="str">
-            <v>FBA79974</v>
-          </cell>
-          <cell r="C149" t="str">
-            <v>B0GD8JSPB1</v>
-          </cell>
-          <cell r="E149" t="str">
-            <v>AM-S1 Bookshelf Speaker</v>
-          </cell>
-        </row>
-        <row r="150">
-          <cell r="B150" t="str">
-            <v>FBA79653</v>
-          </cell>
-          <cell r="C150" t="str">
-            <v>B0DN6LJZBR</v>
-          </cell>
-          <cell r="E150" t="str">
-            <v>AM-C45 Pro</v>
-          </cell>
-        </row>
-        <row r="151">
-          <cell r="B151" t="str">
-            <v>FBA79654</v>
-          </cell>
-          <cell r="C151" t="str">
-            <v>B0DN6MNS1X</v>
-          </cell>
-          <cell r="E151" t="str">
-            <v>AM-C11 Pro</v>
-          </cell>
-        </row>
-        <row r="152">
-          <cell r="B152" t="str">
-            <v>FBA79655</v>
-          </cell>
-          <cell r="C152" t="str">
-            <v>B0DN6PFWNK</v>
-          </cell>
-          <cell r="E152" t="str">
-            <v>AM-C44 Pro</v>
-          </cell>
-        </row>
-        <row r="153">
-          <cell r="B153" t="str">
-            <v>FBA79694</v>
-          </cell>
-          <cell r="C153" t="str">
-            <v>B0DT6T6N6B</v>
-          </cell>
-          <cell r="E153" t="str">
-            <v>AA-26</v>
-          </cell>
-        </row>
-        <row r="154">
-          <cell r="B154" t="str">
-            <v>FBM79708</v>
-          </cell>
-          <cell r="C154" t="str">
-            <v>B0FJS7JZ4V</v>
-          </cell>
-          <cell r="E154" t="str">
-            <v>SB-01</v>
-          </cell>
-        </row>
-        <row r="155">
-          <cell r="B155" t="str">
-            <v>FBM79708</v>
-          </cell>
-          <cell r="C155" t="str">
-            <v>B0FFB6YJM1</v>
-          </cell>
-          <cell r="E155" t="str">
-            <v>SB-01</v>
-          </cell>
-        </row>
-        <row r="156">
-          <cell r="B156" t="str">
-            <v>FBA79783</v>
-          </cell>
-          <cell r="C156" t="str">
-            <v>B0FF9R3GKK</v>
-          </cell>
-          <cell r="E156" t="str">
-            <v>AM-C47</v>
-          </cell>
-        </row>
-        <row r="157">
-          <cell r="B157" t="str">
-            <v>FBA79813</v>
-          </cell>
-          <cell r="C157" t="str">
-            <v>B0FG88HVQ8</v>
-          </cell>
-          <cell r="E157" t="str">
-            <v>AH-50</v>
-          </cell>
-        </row>
-        <row r="158">
-          <cell r="B158" t="str">
-            <v>FBA79814</v>
-          </cell>
-          <cell r="C158" t="str">
-            <v>B0GNM35G8X</v>
-          </cell>
-          <cell r="E158" t="str">
-            <v>AH-50 Ear Cushion</v>
-          </cell>
-        </row>
-        <row r="159">
-          <cell r="B159" t="str">
-            <v>FBA79815</v>
-          </cell>
-          <cell r="C159" t="str">
-            <v>B0FPR7VFCH</v>
-          </cell>
-          <cell r="E159" t="str">
-            <v>AM-W19</v>
-          </cell>
-        </row>
-        <row r="160">
-          <cell r="B160" t="str">
-            <v>FBA79967</v>
-          </cell>
-          <cell r="C160" t="str">
-            <v>B0G2C2RCXN</v>
-          </cell>
-          <cell r="E160" t="str">
-            <v>AM-W19 Duplicate</v>
-          </cell>
-        </row>
-        <row r="161">
-          <cell r="B161" t="str">
-            <v>FBA79816</v>
-          </cell>
-          <cell r="C161" t="str">
-            <v>B0FPR962YS</v>
-          </cell>
-          <cell r="E161" t="str">
-            <v>AM-W22</v>
-          </cell>
-        </row>
-        <row r="162">
-          <cell r="B162" t="str">
-            <v>FBA80016</v>
-          </cell>
-          <cell r="C162" t="str">
-            <v>B0GKPXQ8G3</v>
-          </cell>
-          <cell r="E162" t="str">
-            <v>AM-W22 Duplicate</v>
-          </cell>
-        </row>
-        <row r="163">
-          <cell r="B163" t="str">
-            <v>FBA79820</v>
-          </cell>
-          <cell r="C163" t="str">
-            <v>B0FQJWWDVK</v>
-          </cell>
-          <cell r="E163" t="str">
-            <v>AC-3XL</v>
-          </cell>
-        </row>
-        <row r="164">
-          <cell r="B164" t="str">
-            <v>FBA79838</v>
-          </cell>
-          <cell r="C164" t="str">
-            <v>B0FQBX8J17</v>
-          </cell>
-          <cell r="E164" t="str">
-            <v>AH-40 SL</v>
-          </cell>
-        </row>
-        <row r="165">
-          <cell r="B165" t="str">
-            <v>FBA79839</v>
-          </cell>
-          <cell r="C165" t="str">
-            <v>B0FQBXS6Y2</v>
-          </cell>
-          <cell r="E165" t="str">
-            <v>AH-45 BK</v>
-          </cell>
-        </row>
-        <row r="166">
-          <cell r="B166" t="str">
-            <v>FBA79840</v>
-          </cell>
-          <cell r="C166" t="str">
-            <v>B0FQBWV1ST</v>
-          </cell>
-          <cell r="E166" t="str">
-            <v>AH-60 RD</v>
-          </cell>
-        </row>
-        <row r="167">
-          <cell r="B167" t="str">
-            <v>FBA79841</v>
-          </cell>
-          <cell r="C167" t="str">
-            <v>B0FQBTRM28</v>
-          </cell>
-          <cell r="E167" t="str">
-            <v>AH-60 BL</v>
-          </cell>
-        </row>
-        <row r="168">
-          <cell r="B168" t="str">
-            <v>FBA79842</v>
-          </cell>
-          <cell r="C168" t="str">
-            <v>B0G4DNF8RZ</v>
-          </cell>
-          <cell r="E168" t="str">
-            <v>AM-C48</v>
-          </cell>
-        </row>
-        <row r="169">
-          <cell r="B169" t="str">
-            <v>FBA79821</v>
-          </cell>
-          <cell r="C169" t="str">
-            <v>B0FJ2JJZL3</v>
-          </cell>
-          <cell r="E169" t="str">
-            <v>UB-01</v>
-          </cell>
-        </row>
-        <row r="170">
-          <cell r="B170" t="str">
-            <v>FBA79822</v>
-          </cell>
-          <cell r="C170" t="str">
-            <v>B0FJ2J6MTF</v>
-          </cell>
-          <cell r="E170" t="str">
-            <v>KB-01</v>
-          </cell>
-        </row>
-        <row r="171">
-          <cell r="B171" t="str">
-            <v>FBA79823</v>
-          </cell>
-          <cell r="C171" t="str">
-            <v>B0FJ2HZCVN</v>
-          </cell>
-          <cell r="E171" t="str">
-            <v>PB-01</v>
-          </cell>
-        </row>
-        <row r="172">
-          <cell r="B172" t="str">
-            <v>FBA79824</v>
-          </cell>
-          <cell r="C172" t="str">
-            <v>B0FJ2K95XT</v>
-          </cell>
-          <cell r="E172" t="str">
-            <v>GB-01</v>
-          </cell>
-        </row>
-        <row r="173">
-          <cell r="B173" t="str">
-            <v>FBA79825</v>
-          </cell>
-          <cell r="C173" t="str">
-            <v>B0FJ2DT13L</v>
-          </cell>
-          <cell r="E173" t="str">
-            <v>GB-02</v>
-          </cell>
-        </row>
-        <row r="174">
-          <cell r="B174" t="str">
-            <v>FBA79826</v>
-          </cell>
-          <cell r="C174" t="str">
-            <v>B0FJ2LQT7K</v>
-          </cell>
-          <cell r="E174" t="str">
-            <v>PB-02</v>
-          </cell>
-        </row>
-        <row r="175">
-          <cell r="B175" t="str">
-            <v>FBA79827</v>
-          </cell>
-          <cell r="C175" t="str">
-            <v>B0FJ8S5XJ8</v>
-          </cell>
-          <cell r="E175" t="str">
-            <v>PB-03</v>
-          </cell>
-        </row>
-        <row r="176">
-          <cell r="B176" t="str">
-            <v>FBA79830</v>
-          </cell>
-          <cell r="C176" t="str">
-            <v>B0FJ8TSQK1</v>
-          </cell>
-          <cell r="E176" t="str">
-            <v>GB-03</v>
-          </cell>
-        </row>
-        <row r="177">
-          <cell r="B177" t="str">
-            <v>FBA79831</v>
-          </cell>
-          <cell r="C177" t="str">
-            <v>B0FJ8W5Y9Q</v>
-          </cell>
-          <cell r="E177" t="str">
-            <v>GB-04</v>
-          </cell>
-        </row>
-        <row r="178">
-          <cell r="B178" t="str">
-            <v>FBA79832</v>
-          </cell>
-          <cell r="C178" t="str">
-            <v>B0FJ8S53GW</v>
-          </cell>
-          <cell r="E178" t="str">
-            <v>GB-05</v>
-          </cell>
-        </row>
-        <row r="179">
-          <cell r="B179" t="str">
-            <v>FBA79833</v>
-          </cell>
-          <cell r="C179" t="str">
-            <v>B0FJ8PZ9H7</v>
-          </cell>
-          <cell r="E179" t="str">
-            <v>PB-04</v>
-          </cell>
-        </row>
-        <row r="180">
-          <cell r="B180" t="str">
-            <v>FBA79834</v>
-          </cell>
-          <cell r="C180" t="str">
-            <v>B0FJ8T4WXM</v>
-          </cell>
-          <cell r="E180" t="str">
-            <v>PB-05</v>
-          </cell>
-        </row>
-        <row r="181">
-          <cell r="B181" t="str">
-            <v>FBA79835</v>
-          </cell>
-          <cell r="C181" t="str">
-            <v>B0FJ8TWCQZ</v>
-          </cell>
-          <cell r="E181" t="str">
-            <v>PB-06</v>
-          </cell>
-        </row>
-        <row r="182">
-          <cell r="B182" t="str">
-            <v>FBA79836</v>
-          </cell>
-          <cell r="C182" t="str">
-            <v>B0FJ8Z1W81</v>
-          </cell>
-          <cell r="E182" t="str">
-            <v>PB-07</v>
-          </cell>
-        </row>
-        <row r="183">
-          <cell r="B183" t="str">
-            <v>FBA79844</v>
-          </cell>
-          <cell r="C183" t="str">
-            <v>B0FN7DYB2M</v>
-          </cell>
-          <cell r="E183" t="str">
-            <v>PB-08</v>
-          </cell>
-        </row>
-        <row r="184">
-          <cell r="B184" t="str">
-            <v>FBA79845</v>
-          </cell>
-          <cell r="C184" t="str">
-            <v>B0FN7B3KWS</v>
-          </cell>
-          <cell r="E184" t="str">
-            <v>UB-02</v>
-          </cell>
-        </row>
-        <row r="185">
-          <cell r="B185" t="str">
-            <v>FBA79846</v>
-          </cell>
-          <cell r="C185" t="str">
-            <v>B0FN7C25VS</v>
-          </cell>
-          <cell r="E185" t="str">
-            <v>AM-C11X Pro</v>
-          </cell>
-        </row>
-        <row r="186">
-          <cell r="B186" t="str">
-            <v>FBA79847</v>
-          </cell>
-          <cell r="C186" t="str">
-            <v>B0FN7FYZM3</v>
-          </cell>
-          <cell r="E186" t="str">
-            <v>PB-09</v>
-          </cell>
-        </row>
-        <row r="187">
-          <cell r="B187" t="str">
-            <v>FBA79848</v>
-          </cell>
-          <cell r="C187" t="str">
-            <v>B0GN97RFPR</v>
-          </cell>
-          <cell r="E187" t="str">
-            <v>AM-S2</v>
-          </cell>
-        </row>
-        <row r="188">
-          <cell r="B188" t="str">
-            <v>FBA79904</v>
-          </cell>
-          <cell r="C188" t="str">
-            <v>B0FTVQQVDC</v>
-          </cell>
-          <cell r="E188" t="str">
-            <v>PB-10</v>
-          </cell>
-        </row>
-        <row r="189">
-          <cell r="B189" t="str">
-            <v>FBA79905</v>
-          </cell>
-          <cell r="C189" t="str">
-            <v>B0FTVSH458</v>
-          </cell>
-          <cell r="E189" t="str">
-            <v>PB-11</v>
-          </cell>
-        </row>
-        <row r="190">
-          <cell r="B190" t="str">
-            <v>FBA79906</v>
-          </cell>
-          <cell r="C190" t="str">
-            <v>B0FTVVLNS9</v>
-          </cell>
-          <cell r="E190" t="str">
-            <v>PB-12</v>
-          </cell>
-        </row>
-        <row r="191">
-          <cell r="B191" t="str">
-            <v>FBA79907</v>
-          </cell>
-          <cell r="C191" t="str">
-            <v>B0FTVS34SD</v>
-          </cell>
-          <cell r="E191" t="str">
-            <v>PB-13</v>
-          </cell>
-        </row>
-        <row r="192">
-          <cell r="B192" t="str">
-            <v>FBA79908</v>
-          </cell>
-          <cell r="C192" t="str">
-            <v>B0FTVV1QJY</v>
-          </cell>
-          <cell r="E192" t="str">
-            <v>PB-14</v>
-          </cell>
-        </row>
-        <row r="193">
-          <cell r="B193" t="str">
-            <v>FBA79969</v>
-          </cell>
-          <cell r="C193" t="str">
-            <v>B0G3B677Z5</v>
-          </cell>
-          <cell r="E193" t="str">
-            <v>UB-03</v>
-          </cell>
-        </row>
-        <row r="194">
-          <cell r="B194" t="str">
-            <v>FBA79957</v>
-          </cell>
-          <cell r="C194" t="str">
-            <v>B0G3Q517Y2</v>
-          </cell>
-          <cell r="E194" t="str">
-            <v>AM-W23</v>
-          </cell>
-        </row>
-        <row r="195">
-          <cell r="B195" t="str">
-            <v>FBA79958</v>
-          </cell>
-          <cell r="C195" t="str">
-            <v>B0G3Q59X8C</v>
-          </cell>
-          <cell r="E195" t="str">
-            <v>AM-W24</v>
-          </cell>
-        </row>
-        <row r="196">
-          <cell r="B196" t="str">
-            <v>FBA79961</v>
-          </cell>
-          <cell r="C196" t="str">
-            <v>B0G53H49BS</v>
-          </cell>
-          <cell r="E196" t="str">
-            <v>AI-13</v>
-          </cell>
-        </row>
-        <row r="197">
-          <cell r="B197" t="str">
-            <v>FBA79962</v>
-          </cell>
-          <cell r="C197" t="str">
-            <v>B0G53LZNY3</v>
-          </cell>
-          <cell r="E197" t="str">
-            <v>AM-Mix4 OTG</v>
-          </cell>
-        </row>
-        <row r="198">
-          <cell r="B198" t="str">
-            <v>FBA79963</v>
-          </cell>
-          <cell r="C198" t="str">
-            <v>B0G53CB72D</v>
-          </cell>
-          <cell r="E198" t="str">
-            <v>AM-Pro8</v>
-          </cell>
-        </row>
-        <row r="199">
-          <cell r="B199" t="str">
-            <v>FBA79964</v>
-          </cell>
-          <cell r="C199" t="str">
-            <v>B0G53KWRWH</v>
-          </cell>
-          <cell r="E199" t="str">
-            <v>AM-Pro12</v>
-          </cell>
-        </row>
-        <row r="200">
-          <cell r="B200" t="str">
-            <v>FBA79965</v>
-          </cell>
-          <cell r="C200" t="str">
-            <v>B0G53PRM34</v>
-          </cell>
-          <cell r="E200" t="str">
-            <v>AM-Mix6</v>
-          </cell>
-        </row>
-        <row r="201">
-          <cell r="B201" t="str">
-            <v>FBA79966</v>
-          </cell>
-          <cell r="C201" t="str">
-            <v>B0G53KWRVW</v>
-          </cell>
-          <cell r="E201" t="str">
-            <v>AM-Mix10</v>
-          </cell>
-        </row>
-        <row r="202">
-          <cell r="B202" t="str">
-            <v>FBA79968</v>
-          </cell>
-          <cell r="C202" t="str">
-            <v>B0G53M9258</v>
-          </cell>
-          <cell r="E202" t="str">
-            <v>AI-14</v>
-          </cell>
-        </row>
-        <row r="203">
-          <cell r="B203" t="str">
-            <v>FBA79972</v>
-          </cell>
-          <cell r="C203" t="str">
-            <v>B0GCP1J2HC</v>
-          </cell>
-          <cell r="E203" t="str">
-            <v>M8</v>
-          </cell>
-        </row>
-        <row r="204">
-          <cell r="B204" t="str">
-            <v>FBA80007</v>
-          </cell>
-          <cell r="C204" t="str">
-            <v>B0GN2LHJY4</v>
-          </cell>
-          <cell r="E204" t="str">
-            <v>MT-12</v>
-          </cell>
-        </row>
-        <row r="205">
-          <cell r="B205" t="str">
-            <v>FBA80084</v>
-          </cell>
-          <cell r="E205" t="str">
-            <v>BE-4</v>
-          </cell>
-        </row>
-        <row r="206">
-          <cell r="B206" t="str">
-            <v>FBA80085</v>
-          </cell>
-          <cell r="E206" t="str">
-            <v>M6</v>
-          </cell>
-        </row>
-        <row r="207">
-          <cell r="B207" t="str">
-            <v>FBA79956</v>
-          </cell>
-          <cell r="C207" t="str">
-            <v>B0GMPGNXX3</v>
-          </cell>
-          <cell r="E207" t="str">
-            <v>A3-XLR</v>
-          </cell>
-        </row>
-        <row r="208">
-          <cell r="B208" t="str">
-            <v>FBA80006</v>
-          </cell>
-          <cell r="E208" t="str">
-            <v>A2-XLR</v>
-          </cell>
-        </row>
-        <row r="209">
-          <cell r="B209" t="str">
-            <v>FBA79959</v>
-          </cell>
-          <cell r="C209" t="str">
-            <v>B0G39ZHDYP</v>
-          </cell>
-          <cell r="E209" t="str">
-            <v>AM-W47 Wired</v>
-          </cell>
-        </row>
-        <row r="210">
-          <cell r="B210" t="str">
-            <v xml:space="preserve">FBA79960 </v>
-          </cell>
-          <cell r="C210" t="str">
-            <v>B0G3B152FR</v>
-          </cell>
-          <cell r="E210" t="str">
-            <v>AM-W47 Wireless</v>
-          </cell>
-        </row>
-        <row r="211">
-          <cell r="B211" t="str">
-            <v>FBA79975</v>
-          </cell>
-          <cell r="E211" t="str">
-            <v>AE831</v>
-          </cell>
-        </row>
-        <row r="212">
-          <cell r="B212" t="str">
-            <v>FBA79976</v>
-          </cell>
-          <cell r="E212" t="str">
-            <v>JT-1</v>
-          </cell>
-        </row>
-        <row r="213">
-          <cell r="B213" t="str">
-            <v>FBA79977</v>
-          </cell>
-          <cell r="E213" t="str">
-            <v>BM-320PRO</v>
-          </cell>
-        </row>
-        <row r="214">
-          <cell r="B214" t="str">
-            <v>FBA79979</v>
-          </cell>
-          <cell r="C214" t="str">
-            <v>B0GN8RQJRG</v>
-          </cell>
-          <cell r="E214" t="str">
-            <v>AK-37-B</v>
-          </cell>
-        </row>
-        <row r="215">
-          <cell r="B215" t="str">
-            <v>FBA79980</v>
-          </cell>
-          <cell r="C215" t="str">
-            <v>B0GN8MMKY1</v>
-          </cell>
-          <cell r="E215" t="str">
-            <v>AK-37-W</v>
-          </cell>
-        </row>
-        <row r="216">
-          <cell r="B216" t="str">
-            <v>FBA79981</v>
-          </cell>
-          <cell r="C216" t="str">
-            <v>B0GN8MFDGZ</v>
-          </cell>
-          <cell r="E216" t="str">
-            <v>AK-61 Neo</v>
-          </cell>
-        </row>
-        <row r="217">
-          <cell r="B217" t="str">
-            <v>FBA79982</v>
-          </cell>
-          <cell r="C217" t="str">
-            <v>B0GN8MPYPG</v>
-          </cell>
-          <cell r="E217" t="str">
-            <v>AK-61 Pro</v>
-          </cell>
-        </row>
-        <row r="218">
-          <cell r="B218" t="str">
-            <v>FBA79983</v>
-          </cell>
-          <cell r="C218" t="str">
-            <v>B0GN321RXQ</v>
-          </cell>
-          <cell r="E218" t="str">
-            <v>AM-W48 / AM-S6</v>
-          </cell>
-        </row>
-        <row r="219">
-          <cell r="B219" t="str">
-            <v>FBA79996</v>
-          </cell>
-          <cell r="E219" t="str">
-            <v>AM-C49</v>
-          </cell>
-        </row>
-        <row r="220">
-          <cell r="B220" t="str">
-            <v>FBA79995</v>
-          </cell>
-          <cell r="E220" t="str">
-            <v>AM-C50</v>
-          </cell>
-        </row>
-        <row r="221">
-          <cell r="B221" t="str">
-            <v>FBA79997</v>
-          </cell>
-          <cell r="E221" t="str">
-            <v>W3</v>
-          </cell>
-        </row>
-        <row r="222">
-          <cell r="B222" t="str">
-            <v>FBA79998</v>
-          </cell>
-          <cell r="E222" t="str">
-            <v>W5</v>
-          </cell>
-        </row>
-        <row r="223">
-          <cell r="B223" t="str">
-            <v>FBA79999</v>
-          </cell>
-          <cell r="E223" t="str">
-            <v>JTG800</v>
-          </cell>
-        </row>
-        <row r="224">
-          <cell r="B224" t="str">
-            <v>FBA80000</v>
-          </cell>
-          <cell r="E224" t="str">
-            <v>DP-718H</v>
-          </cell>
-        </row>
-        <row r="225">
-          <cell r="B225" t="str">
-            <v>FBA80001</v>
-          </cell>
-          <cell r="E225" t="str">
-            <v>USB718</v>
-          </cell>
-        </row>
-        <row r="226">
-          <cell r="B226" t="str">
-            <v>FBA80002</v>
-          </cell>
-          <cell r="E226" t="str">
-            <v>AM-W33 Pro</v>
-          </cell>
-        </row>
-        <row r="227">
-          <cell r="B227" t="str">
-            <v>FBA80003</v>
-          </cell>
-          <cell r="E227" t="str">
-            <v>AM-W32 Pro</v>
-          </cell>
-        </row>
-        <row r="228">
-          <cell r="B228" t="str">
-            <v>FBA80004</v>
-          </cell>
-          <cell r="E228" t="str">
-            <v>AM-W36 Pro</v>
-          </cell>
-        </row>
-        <row r="229">
-          <cell r="B229" t="str">
-            <v>FBA80005</v>
-          </cell>
-          <cell r="E229" t="str">
-            <v>T-835</v>
-          </cell>
-        </row>
-        <row r="230">
-          <cell r="B230" t="str">
-            <v>FBA80009</v>
-          </cell>
-          <cell r="E230" t="str">
-            <v>AM-C51</v>
-          </cell>
-        </row>
-        <row r="231">
-          <cell r="B231" t="str">
-            <v>FBA80010</v>
-          </cell>
-          <cell r="E231" t="str">
-            <v>AM-C52</v>
-          </cell>
-        </row>
-        <row r="232">
-          <cell r="B232" t="str">
-            <v>FBA80011</v>
-          </cell>
-          <cell r="E232" t="str">
-            <v>AM-Pro16</v>
-          </cell>
-        </row>
-        <row r="233">
-          <cell r="B233" t="str">
-            <v>FBA80012</v>
-          </cell>
-          <cell r="E233" t="str">
-            <v>AM-Pro24</v>
-          </cell>
-        </row>
-        <row r="234">
-          <cell r="B234" t="str">
-            <v>FBA80013</v>
-          </cell>
-          <cell r="E234" t="str">
-            <v>XM-16</v>
-          </cell>
-        </row>
-        <row r="235">
-          <cell r="B235" t="str">
-            <v>FBA80014</v>
-          </cell>
-          <cell r="E235" t="str">
-            <v>XM-24</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11378,12 +8826,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:I843"/>
+  <dimension ref="A1:I833"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.109375" style="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.5546875" style="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.88671875" style="13" bestFit="1" customWidth="1"/>
@@ -12990,13 +10438,13 @@
     </row>
     <row r="56" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>2703</v>
+        <v>2702</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>2703</v>
+        <v>2702</v>
       </c>
       <c r="C56" t="s">
-        <v>2702</v>
+        <v>2701</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>6</v>
@@ -13715,13 +11163,13 @@
     </row>
     <row r="81" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
+        <v>2703</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>2703</v>
+      </c>
+      <c r="C81" t="s">
         <v>2704</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>2704</v>
-      </c>
-      <c r="C81" t="s">
-        <v>2705</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>6</v>
@@ -16053,8 +13501,8 @@
         <v>543</v>
       </c>
       <c r="B164" s="2"/>
-      <c r="C164" s="2" t="s">
-        <v>747</v>
+      <c r="C164" t="s">
+        <v>2700</v>
       </c>
       <c r="D164" s="2" t="s">
         <v>523</v>
@@ -16078,8 +13526,8 @@
         <v>544</v>
       </c>
       <c r="B165" s="2"/>
-      <c r="C165" s="2" t="s">
-        <v>747</v>
+      <c r="C165" t="s">
+        <v>2705</v>
       </c>
       <c r="D165" s="2" t="s">
         <v>523</v>
@@ -16103,8 +13551,8 @@
         <v>545</v>
       </c>
       <c r="B166" s="2"/>
-      <c r="C166" s="2" t="s">
-        <v>747</v>
+      <c r="C166" t="s">
+        <v>2706</v>
       </c>
       <c r="D166" s="2" t="s">
         <v>523</v>
@@ -16128,8 +13576,8 @@
         <v>546</v>
       </c>
       <c r="B167" s="2"/>
-      <c r="C167" s="2" t="s">
-        <v>747</v>
+      <c r="C167" t="s">
+        <v>2699</v>
       </c>
       <c r="D167" s="2" t="s">
         <v>523</v>
@@ -18179,7 +15627,7 @@
       </c>
       <c r="B249" s="2"/>
       <c r="C249" t="s">
-        <v>2708</v>
+        <v>2707</v>
       </c>
       <c r="D249" s="2" t="s">
         <v>523</v>
@@ -29990,205 +27438,50 @@
         <v>2671</v>
       </c>
     </row>
-    <row r="834" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A834" s="17" t="s">
-        <v>546</v>
-      </c>
-      <c r="C834" t="s">
-        <v>2699</v>
-      </c>
-      <c r="D834" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E834" s="17" t="s">
-        <v>931</v>
-      </c>
-      <c r="F834" s="17" t="s">
-        <v>2701</v>
-      </c>
-    </row>
-    <row r="835" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A835" s="17" t="s">
-        <v>543</v>
-      </c>
-      <c r="C835" t="s">
-        <v>2700</v>
-      </c>
-      <c r="D835" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E835" s="17" t="s">
-        <v>928</v>
-      </c>
-      <c r="F835" s="17" t="s">
-        <v>2701</v>
-      </c>
-    </row>
-    <row r="836" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A836" s="17" t="s">
-        <v>576</v>
-      </c>
-      <c r="C836" s="17" t="str">
-        <f>_xlfn.XLOOKUP(A836,[1]Main!$B:$B,[1]Main!$C:$C)</f>
-        <v>B0FJ2JJZL3</v>
-      </c>
-      <c r="D836" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E836" s="17" t="str">
-        <f>_xlfn.XLOOKUP(C836,[1]Main!$C:$C,[1]Main!$E:$E)</f>
-        <v>UB-01</v>
-      </c>
-      <c r="F836" s="17" t="s">
-        <v>1135</v>
-      </c>
-    </row>
-    <row r="837" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A837" s="13" t="s">
-        <v>692</v>
-      </c>
-      <c r="C837" s="17" t="str">
-        <f>_xlfn.XLOOKUP(A837,[1]Main!$B:$B,[1]Main!$C:$C)</f>
-        <v>B0FN7B3KWS</v>
-      </c>
-      <c r="D837" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E837" s="17" t="str">
-        <f>_xlfn.XLOOKUP(C837,[1]Main!$C:$C,[1]Main!$E:$E)</f>
-        <v>UB-02</v>
-      </c>
-      <c r="F837" s="17" t="s">
-        <v>1135</v>
-      </c>
-    </row>
-    <row r="838" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A838" s="17" t="s">
-        <v>544</v>
-      </c>
-      <c r="C838" t="s">
-        <v>2706</v>
-      </c>
-      <c r="D838" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E838" s="17" t="s">
-        <v>929</v>
-      </c>
-    </row>
-    <row r="839" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A839" s="17" t="s">
-        <v>545</v>
-      </c>
-      <c r="C839" t="s">
-        <v>2707</v>
-      </c>
-      <c r="D839" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E839" s="17" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="840" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A840" s="13" t="s">
-        <v>543</v>
-      </c>
-      <c r="C840" s="13" t="s">
-        <v>2700</v>
-      </c>
-      <c r="D840" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E840" s="13" t="s">
-        <v>928</v>
-      </c>
-    </row>
-    <row r="841" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A841" s="13" t="s">
-        <v>544</v>
-      </c>
-      <c r="C841" s="13" t="s">
-        <v>2706</v>
-      </c>
-      <c r="D841" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E841" s="13" t="s">
-        <v>929</v>
-      </c>
-    </row>
-    <row r="842" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A842" s="13" t="s">
-        <v>545</v>
-      </c>
-      <c r="C842" s="13" t="s">
-        <v>2707</v>
-      </c>
-      <c r="D842" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E842" s="13" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="843" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A843" s="13" t="s">
-        <v>546</v>
-      </c>
-      <c r="C843" s="13" t="s">
-        <v>2699</v>
-      </c>
-      <c r="D843" s="13" t="s">
-        <v>523</v>
-      </c>
-      <c r="E843" s="13" t="s">
-        <v>931</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="16" priority="67"/>
+  <autoFilter ref="A1:I833" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}"/>
+  <conditionalFormatting sqref="A92">
+    <cfRule type="duplicateValues" dxfId="16" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="59"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A92">
-    <cfRule type="duplicateValues" dxfId="15" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="59"/>
+  <conditionalFormatting sqref="B56 A93:A104 A106:A122 A31:A91 A21:A29 B81 A2:A19">
+    <cfRule type="duplicateValues" dxfId="14" priority="76"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A93:A104 A106:A122 A2:A19 A31:A91 A21:A29 B56 B81">
-    <cfRule type="duplicateValues" dxfId="13" priority="68"/>
+  <conditionalFormatting sqref="A123:B123">
+    <cfRule type="duplicateValues" dxfId="13" priority="50"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A124:B140">
+    <cfRule type="duplicateValues" dxfId="12" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A141:A144">
-    <cfRule type="duplicateValues" dxfId="12" priority="49"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A123:B123">
-    <cfRule type="duplicateValues" dxfId="11" priority="50"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A124:B140">
-    <cfRule type="duplicateValues" dxfId="10" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="9" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="7" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C92">
-    <cfRule type="duplicateValues" dxfId="6" priority="54"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C95">
-    <cfRule type="duplicateValues" dxfId="4" priority="51"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="2" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E124:E140">
-    <cfRule type="duplicateValues" dxfId="1" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E141">
-    <cfRule type="duplicateValues" dxfId="0" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="47"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="duplicateValues" dxfId="0" priority="86"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A121" r:id="rId1" display="https://sellercentral.amazon.in/skucentral?mSku=FBA79849&amp;condition=New&amp;ref_=myp_skuc" xr:uid="{F5F7F880-2E3B-44E2-BABD-2E8055A5AAE6}"/>

</xml_diff>

<commit_message>
data: Week 15 sales data, updated SKU master, sales snapshot, AI context
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BE5D17-2B57-487B-A798-CD2069CA5053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C3398A-461E-45E0-9F92-253344F73178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -8410,40 +8410,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -8548,6 +8514,40 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -29211,67 +29211,67 @@
     <cfRule type="duplicateValues" dxfId="33" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A92">
-    <cfRule type="duplicateValues" dxfId="32" priority="75"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A141:A144">
     <cfRule type="duplicateValues" dxfId="30" priority="66"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A836:A839">
+    <cfRule type="duplicateValues" dxfId="29" priority="17"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A123:B123">
-    <cfRule type="duplicateValues" dxfId="29" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A124:B140">
-    <cfRule type="duplicateValues" dxfId="28" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56 A93:A104 A106:A122 A31:A91 A21:A29 B81 A2:A19">
-    <cfRule type="duplicateValues" dxfId="27" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="26" priority="73"/>
     <cfRule type="duplicateValues" dxfId="25" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="24" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C92">
-    <cfRule type="duplicateValues" dxfId="23" priority="71"/>
     <cfRule type="duplicateValues" dxfId="22" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C95">
-    <cfRule type="duplicateValues" dxfId="21" priority="68"/>
     <cfRule type="duplicateValues" dxfId="20" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="68"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E1">
+    <cfRule type="duplicateValues" dxfId="18" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E124:E140">
-    <cfRule type="duplicateValues" dxfId="19" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="63"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E141">
-    <cfRule type="duplicateValues" dxfId="18" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="64"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A836:A839">
-    <cfRule type="duplicateValues" dxfId="17" priority="17"/>
+  <conditionalFormatting sqref="E400">
+    <cfRule type="duplicateValues" dxfId="15" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E836:E839">
-    <cfRule type="duplicateValues" dxfId="16" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="16" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E400">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="8" stopIfTrue="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="0" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="15" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A121" r:id="rId1" display="https://sellercentral.amazon.in/skucentral?mSku=FBA79849&amp;condition=New&amp;ref_=myp_skuc" xr:uid="{F5F7F880-2E3B-44E2-BABD-2E8055A5AAE6}"/>

</xml_diff>

<commit_message>
Update weekly report data and add week 17 files
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E36D84-6401-46A3-A6B2-46D2007E0138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60FA1A5C-2B51-465A-B1FF-5DF497804438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4973" uniqueCount="2728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4973" uniqueCount="2729">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -8221,6 +8221,9 @@
   </si>
   <si>
     <t>FBP79569</t>
+  </si>
+  <si>
+    <t>B0GV154XPQ</t>
   </si>
 </sst>
 </file>
@@ -8412,30 +8415,6 @@
   <dxfs count="34">
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -8560,6 +8539,30 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -18166,7 +18169,7 @@
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="2" t="s">
-        <v>747</v>
+        <v>2728</v>
       </c>
       <c r="D340" s="2" t="s">
         <v>523</v>
@@ -29265,8 +29268,8 @@
     <cfRule type="duplicateValues" dxfId="33" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A93">
-    <cfRule type="duplicateValues" dxfId="32" priority="75"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A142:A145">
     <cfRule type="duplicateValues" dxfId="30" priority="66"/>
@@ -29284,19 +29287,19 @@
     <cfRule type="duplicateValues" dxfId="26" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="25" priority="73"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B123">
     <cfRule type="duplicateValues" dxfId="23" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C93">
-    <cfRule type="duplicateValues" dxfId="22" priority="71"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C96">
-    <cfRule type="duplicateValues" dxfId="20" priority="68"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
     <cfRule type="duplicateValues" dxfId="18" priority="104"/>
@@ -29308,24 +29311,24 @@
     <cfRule type="duplicateValues" dxfId="16" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E401">
-    <cfRule type="duplicateValues" dxfId="15" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
     <cfRule type="duplicateValues" dxfId="11" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="8" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E837:E840">
-    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="15" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A122" r:id="rId1" display="https://sellercentral.amazon.in/skucentral?mSku=FBA79849&amp;condition=New&amp;ref_=myp_skuc" xr:uid="{F5F7F880-2E3B-44E2-BABD-2E8055A5AAE6}"/>

</xml_diff>

<commit_message>
data: sku_master — fill in AM-Pro16 / AM-Pro24 categories
AM-Pro16 → Audio Mixer / 16 Channel Mixer
AM-Pro24 → Audio Mixer / 24 Channel Mixer
(NLC still pending for both — operator will fill in next.)

Restored from sku_master1.xlsx that Excel accidentally created via
Save-As; copied back over the canonical sku_master.xlsx so
load_all_inventory() picks up the new categories.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194FE2E4-0673-40F3-A71F-CFD349A2C73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BAFB67-2ABB-4D1F-9E82-11318C988AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$841</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$868</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4973" uniqueCount="2729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5121" uniqueCount="2817">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -8217,13 +8217,277 @@
     <t>B0D86Y2V7V</t>
   </si>
   <si>
-    <t>B0G1YKMFWT</t>
-  </si>
-  <si>
-    <t>FBP79569</t>
-  </si>
-  <si>
     <t>B0GV154XPQ</t>
+  </si>
+  <si>
+    <t>MK9146</t>
+  </si>
+  <si>
+    <t>AX4611</t>
+  </si>
+  <si>
+    <t>AX2761</t>
+  </si>
+  <si>
+    <t>AX5385</t>
+  </si>
+  <si>
+    <t>AX5616</t>
+  </si>
+  <si>
+    <t>FS6062</t>
+  </si>
+  <si>
+    <t>ES5362</t>
+  </si>
+  <si>
+    <t>AR11673</t>
+  </si>
+  <si>
+    <t>AR11692</t>
+  </si>
+  <si>
+    <t>MK4967</t>
+  </si>
+  <si>
+    <t>DZ2234</t>
+  </si>
+  <si>
+    <t>AR11755</t>
+  </si>
+  <si>
+    <t>ES5455</t>
+  </si>
+  <si>
+    <t>MK7570SET</t>
+  </si>
+  <si>
+    <t>MK7582</t>
+  </si>
+  <si>
+    <t>AX1746</t>
+  </si>
+  <si>
+    <t>FS5665</t>
+  </si>
+  <si>
+    <t>FS5447</t>
+  </si>
+  <si>
+    <t>MK7303</t>
+  </si>
+  <si>
+    <t>ME3154</t>
+  </si>
+  <si>
+    <t>AX1350</t>
+  </si>
+  <si>
+    <t>FS5151</t>
+  </si>
+  <si>
+    <t>DZ4548</t>
+  </si>
+  <si>
+    <t>AR11589</t>
+  </si>
+  <si>
+    <t>AR11606</t>
+  </si>
+  <si>
+    <t>MK4823</t>
+  </si>
+  <si>
+    <t>MK9165</t>
+  </si>
+  <si>
+    <t>AX4614</t>
+  </si>
+  <si>
+    <t>FBA79136</t>
+  </si>
+  <si>
+    <t>B0CFVK4PYT</t>
+  </si>
+  <si>
+    <t>FBA79286</t>
+  </si>
+  <si>
+    <t>B0CR5G3NRL</t>
+  </si>
+  <si>
+    <t>FBA79321</t>
+  </si>
+  <si>
+    <t>B0CR5JQFD5</t>
+  </si>
+  <si>
+    <t>FBA79407</t>
+  </si>
+  <si>
+    <t>B0CWR5S3R7</t>
+  </si>
+  <si>
+    <t>FBA79408</t>
+  </si>
+  <si>
+    <t>B0CYN8F826</t>
+  </si>
+  <si>
+    <t>FBA79419</t>
+  </si>
+  <si>
+    <t>B0CZSF6LVY</t>
+  </si>
+  <si>
+    <t>FBA79528</t>
+  </si>
+  <si>
+    <t>B0D93652ZY</t>
+  </si>
+  <si>
+    <t>FBA79726</t>
+  </si>
+  <si>
+    <t>B0DT2S2Y7F</t>
+  </si>
+  <si>
+    <t>FBA79858</t>
+  </si>
+  <si>
+    <t>B0FFJ4N8BK</t>
+  </si>
+  <si>
+    <t>FBA79947</t>
+  </si>
+  <si>
+    <t>B0FS6N1YT5</t>
+  </si>
+  <si>
+    <t>FBA80035</t>
+  </si>
+  <si>
+    <t>B07SV6Q9QX</t>
+  </si>
+  <si>
+    <t>FBA80038</t>
+  </si>
+  <si>
+    <t>B0GDJJ86QY</t>
+  </si>
+  <si>
+    <t>FBA80041</t>
+  </si>
+  <si>
+    <t>B0GF72VQSX</t>
+  </si>
+  <si>
+    <t>FBA80051</t>
+  </si>
+  <si>
+    <t>B0GF7BSTKP</t>
+  </si>
+  <si>
+    <t>FBA80053</t>
+  </si>
+  <si>
+    <t>B0GF73VZZ2</t>
+  </si>
+  <si>
+    <t>FBA80095</t>
+  </si>
+  <si>
+    <t>B0CHXGWVZJ</t>
+  </si>
+  <si>
+    <t>FBA80096</t>
+  </si>
+  <si>
+    <t>B07WQ9WRJ9</t>
+  </si>
+  <si>
+    <t>FBO67237</t>
+  </si>
+  <si>
+    <t>B079D8QRRL</t>
+  </si>
+  <si>
+    <t>FBO76805</t>
+  </si>
+  <si>
+    <t>B0BG17DJQS</t>
+  </si>
+  <si>
+    <t>FBO76876</t>
+  </si>
+  <si>
+    <t>B0769YW2KN</t>
+  </si>
+  <si>
+    <t>FBO77014</t>
+  </si>
+  <si>
+    <t>B00CJ06DYG</t>
+  </si>
+  <si>
+    <t>FBS66987</t>
+  </si>
+  <si>
+    <t>B017SN1OI8</t>
+  </si>
+  <si>
+    <t>FBS74343</t>
+  </si>
+  <si>
+    <t>B08SW1LBDF</t>
+  </si>
+  <si>
+    <t>FBS79303</t>
+  </si>
+  <si>
+    <t>B0CR5RZRMH</t>
+  </si>
+  <si>
+    <t>FBS79417</t>
+  </si>
+  <si>
+    <t>B0CYNH9X11</t>
+  </si>
+  <si>
+    <t>FBS79424</t>
+  </si>
+  <si>
+    <t>B0CZ9BTN24</t>
+  </si>
+  <si>
+    <t>FBS79428</t>
+  </si>
+  <si>
+    <t>B0CZ93BN92</t>
+  </si>
+  <si>
+    <t>FBS79516</t>
+  </si>
+  <si>
+    <t>B0D85F9QCK</t>
+  </si>
+  <si>
+    <t>Headphone</t>
+  </si>
+  <si>
+    <t>Audio Mixer</t>
+  </si>
+  <si>
+    <t>16 Channel Mixer</t>
+  </si>
+  <si>
+    <t>24 Channel Mixer</t>
+  </si>
+  <si>
+    <t>16 Channel Mixer With Carry Case</t>
+  </si>
+  <si>
+    <t>24 Channel Mixer With Carry Case</t>
   </si>
 </sst>
 </file>
@@ -8415,6 +8679,30 @@
   <dxfs count="34">
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -8539,30 +8827,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -9091,7 +9355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:I841"/>
+  <dimension ref="A1:I868"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="13" bestFit="1" customWidth="1"/>
@@ -18169,7 +18433,7 @@
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="2" t="s">
-        <v>2728</v>
+        <v>2726</v>
       </c>
       <c r="D340" s="2" t="s">
         <v>523</v>
@@ -29148,8 +29412,12 @@
       <c r="E835" s="22" t="s">
         <v>2698</v>
       </c>
-      <c r="F835" s="2"/>
-      <c r="G835" s="2"/>
+      <c r="F835" s="2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="G835" s="2" t="s">
+        <v>2811</v>
+      </c>
       <c r="H835" s="2"/>
       <c r="I835" s="11"/>
     </row>
@@ -29167,8 +29435,12 @@
       <c r="E836" s="22" t="s">
         <v>2699</v>
       </c>
-      <c r="F836" s="2"/>
-      <c r="G836" s="2"/>
+      <c r="F836" s="2" t="s">
+        <v>2811</v>
+      </c>
+      <c r="G836" s="2" t="s">
+        <v>2811</v>
+      </c>
       <c r="H836" s="2"/>
       <c r="I836" s="11"/>
     </row>
@@ -29186,8 +29458,12 @@
       <c r="E837" s="19" t="s">
         <v>2709</v>
       </c>
-      <c r="F837" s="2"/>
-      <c r="G837" s="2"/>
+      <c r="F837" s="2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="G837" s="2" t="s">
+        <v>2813</v>
+      </c>
       <c r="H837" s="2"/>
       <c r="I837" s="11"/>
     </row>
@@ -29205,8 +29481,12 @@
       <c r="E838" s="19" t="s">
         <v>2710</v>
       </c>
-      <c r="F838" s="2"/>
-      <c r="G838" s="2"/>
+      <c r="F838" s="2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="G838" s="2" t="s">
+        <v>2814</v>
+      </c>
       <c r="H838" s="2"/>
       <c r="I838" s="11"/>
     </row>
@@ -29224,8 +29504,12 @@
       <c r="E839" s="19" t="s">
         <v>2711</v>
       </c>
-      <c r="F839" s="2"/>
-      <c r="G839" s="2"/>
+      <c r="F839" s="2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="G839" s="2" t="s">
+        <v>2815</v>
+      </c>
       <c r="H839" s="2"/>
       <c r="I839" s="11"/>
     </row>
@@ -29243,32 +29527,499 @@
       <c r="E840" s="19" t="s">
         <v>2712</v>
       </c>
-      <c r="F840" s="2"/>
-      <c r="G840" s="2"/>
+      <c r="F840" s="2" t="s">
+        <v>2812</v>
+      </c>
+      <c r="G840" s="2" t="s">
+        <v>2816</v>
+      </c>
       <c r="H840" s="2"/>
       <c r="I840" s="11"/>
     </row>
     <row r="841" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A841" s="13" t="s">
+        <v>2755</v>
+      </c>
+      <c r="C841" s="13" t="s">
+        <v>2756</v>
+      </c>
+      <c r="D841" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E841" s="13" t="s">
         <v>2727</v>
       </c>
-      <c r="C841" s="13" t="s">
-        <v>2726</v>
-      </c>
-      <c r="D841" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="E841" s="13" t="s">
-        <v>331</v>
+      <c r="F841" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="842" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A842" s="13" t="s">
+        <v>2757</v>
+      </c>
+      <c r="C842" s="13" t="s">
+        <v>2758</v>
+      </c>
+      <c r="D842" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E842" s="13" t="s">
+        <v>2728</v>
+      </c>
+      <c r="F842" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="843" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A843" s="13" t="s">
+        <v>2759</v>
+      </c>
+      <c r="C843" s="13" t="s">
+        <v>2760</v>
+      </c>
+      <c r="D843" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E843" s="13" t="s">
+        <v>2729</v>
+      </c>
+      <c r="F843" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="844" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A844" s="13" t="s">
+        <v>2761</v>
+      </c>
+      <c r="C844" s="13" t="s">
+        <v>2762</v>
+      </c>
+      <c r="D844" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E844" s="13" t="s">
+        <v>2730</v>
+      </c>
+      <c r="F844" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="845" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A845" s="13" t="s">
+        <v>2763</v>
+      </c>
+      <c r="C845" s="13" t="s">
+        <v>2764</v>
+      </c>
+      <c r="D845" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E845" s="13" t="s">
+        <v>2731</v>
+      </c>
+      <c r="F845" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="846" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A846" s="13" t="s">
+        <v>2765</v>
+      </c>
+      <c r="C846" s="13" t="s">
+        <v>2766</v>
+      </c>
+      <c r="D846" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E846" s="13" t="s">
+        <v>2732</v>
+      </c>
+      <c r="F846" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="847" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A847" s="13" t="s">
+        <v>2767</v>
+      </c>
+      <c r="C847" s="13" t="s">
+        <v>2768</v>
+      </c>
+      <c r="D847" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E847" s="13" t="s">
+        <v>2733</v>
+      </c>
+      <c r="F847" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="848" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A848" s="13" t="s">
+        <v>2769</v>
+      </c>
+      <c r="C848" s="13" t="s">
+        <v>2770</v>
+      </c>
+      <c r="D848" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E848" s="13" t="s">
+        <v>2734</v>
+      </c>
+      <c r="F848" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="849" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A849" s="13" t="s">
+        <v>2771</v>
+      </c>
+      <c r="C849" s="13" t="s">
+        <v>2772</v>
+      </c>
+      <c r="D849" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E849" s="13" t="s">
+        <v>2735</v>
+      </c>
+      <c r="F849" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="850" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A850" s="13" t="s">
+        <v>2773</v>
+      </c>
+      <c r="C850" s="13" t="s">
+        <v>2774</v>
+      </c>
+      <c r="D850" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E850" s="13" t="s">
+        <v>2736</v>
+      </c>
+      <c r="F850" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="851" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A851" s="13" t="s">
+        <v>2775</v>
+      </c>
+      <c r="C851" s="13" t="s">
+        <v>2776</v>
+      </c>
+      <c r="D851" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E851" s="13" t="s">
+        <v>2737</v>
+      </c>
+      <c r="F851" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="852" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A852" s="13" t="s">
+        <v>2777</v>
+      </c>
+      <c r="C852" s="13" t="s">
+        <v>2778</v>
+      </c>
+      <c r="D852" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E852" s="13" t="s">
+        <v>2738</v>
+      </c>
+      <c r="F852" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="853" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A853" s="13" t="s">
+        <v>2779</v>
+      </c>
+      <c r="C853" s="13" t="s">
+        <v>2780</v>
+      </c>
+      <c r="D853" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E853" s="13" t="s">
+        <v>2739</v>
+      </c>
+      <c r="F853" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="854" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A854" s="13" t="s">
+        <v>2781</v>
+      </c>
+      <c r="C854" s="13" t="s">
+        <v>2782</v>
+      </c>
+      <c r="D854" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E854" s="13" t="s">
+        <v>2740</v>
+      </c>
+      <c r="F854" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="855" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A855" s="13" t="s">
+        <v>2783</v>
+      </c>
+      <c r="C855" s="13" t="s">
+        <v>2784</v>
+      </c>
+      <c r="D855" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E855" s="13" t="s">
+        <v>2741</v>
+      </c>
+      <c r="F855" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="856" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A856" s="13" t="s">
+        <v>2785</v>
+      </c>
+      <c r="C856" s="13" t="s">
+        <v>2786</v>
+      </c>
+      <c r="D856" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E856" s="13" t="s">
+        <v>2742</v>
+      </c>
+      <c r="F856" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="857" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A857" s="13" t="s">
+        <v>2787</v>
+      </c>
+      <c r="C857" s="13" t="s">
+        <v>2788</v>
+      </c>
+      <c r="D857" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E857" s="13" t="s">
+        <v>2743</v>
+      </c>
+      <c r="F857" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="858" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A858" s="13" t="s">
+        <v>2789</v>
+      </c>
+      <c r="C858" s="13" t="s">
+        <v>2790</v>
+      </c>
+      <c r="D858" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E858" s="13" t="s">
+        <v>2744</v>
+      </c>
+      <c r="F858" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="859" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A859" s="13" t="s">
+        <v>2791</v>
+      </c>
+      <c r="C859" s="13" t="s">
+        <v>2792</v>
+      </c>
+      <c r="D859" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E859" s="13" t="s">
+        <v>2745</v>
+      </c>
+      <c r="F859" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="860" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A860" s="13" t="s">
+        <v>2793</v>
+      </c>
+      <c r="C860" s="13" t="s">
+        <v>2794</v>
+      </c>
+      <c r="D860" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E860" s="13" t="s">
+        <v>2746</v>
+      </c>
+      <c r="F860" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="861" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A861" s="13" t="s">
+        <v>2795</v>
+      </c>
+      <c r="C861" s="13" t="s">
+        <v>2796</v>
+      </c>
+      <c r="D861" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E861" s="13" t="s">
+        <v>2747</v>
+      </c>
+      <c r="F861" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="862" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A862" s="13" t="s">
+        <v>2797</v>
+      </c>
+      <c r="C862" s="13" t="s">
+        <v>2798</v>
+      </c>
+      <c r="D862" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E862" s="13" t="s">
+        <v>2748</v>
+      </c>
+      <c r="F862" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="863" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A863" s="13" t="s">
+        <v>2799</v>
+      </c>
+      <c r="C863" s="13" t="s">
+        <v>2800</v>
+      </c>
+      <c r="D863" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E863" s="13" t="s">
+        <v>2749</v>
+      </c>
+      <c r="F863" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="864" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A864" s="13" t="s">
+        <v>2801</v>
+      </c>
+      <c r="C864" s="13" t="s">
+        <v>2802</v>
+      </c>
+      <c r="D864" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E864" s="13" t="s">
+        <v>2750</v>
+      </c>
+      <c r="F864" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="865" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A865" s="13" t="s">
+        <v>2803</v>
+      </c>
+      <c r="C865" s="13" t="s">
+        <v>2804</v>
+      </c>
+      <c r="D865" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E865" s="13" t="s">
+        <v>2751</v>
+      </c>
+      <c r="F865" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="866" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A866" s="13" t="s">
+        <v>2805</v>
+      </c>
+      <c r="C866" s="13" t="s">
+        <v>2806</v>
+      </c>
+      <c r="D866" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E866" s="13" t="s">
+        <v>2752</v>
+      </c>
+      <c r="F866" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="867" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A867" s="13" t="s">
+        <v>2807</v>
+      </c>
+      <c r="C867" s="13" t="s">
+        <v>2808</v>
+      </c>
+      <c r="D867" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E867" s="13" t="s">
+        <v>2753</v>
+      </c>
+      <c r="F867" s="13" t="s">
+        <v>2661</v>
+      </c>
+    </row>
+    <row r="868" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A868" s="13" t="s">
+        <v>2809</v>
+      </c>
+      <c r="C868" s="13" t="s">
+        <v>2810</v>
+      </c>
+      <c r="D868" s="13" t="s">
+        <v>2660</v>
+      </c>
+      <c r="E868" s="13" t="s">
+        <v>2754</v>
+      </c>
+      <c r="F868" s="13" t="s">
+        <v>2661</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I868" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}"/>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="33" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A93">
-    <cfRule type="duplicateValues" dxfId="32" priority="76"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A142:A145">
     <cfRule type="duplicateValues" dxfId="30" priority="66"/>
@@ -29286,19 +30037,19 @@
     <cfRule type="duplicateValues" dxfId="26" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="25" priority="74"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B123">
     <cfRule type="duplicateValues" dxfId="23" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C93">
-    <cfRule type="duplicateValues" dxfId="22" priority="72"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C96">
-    <cfRule type="duplicateValues" dxfId="20" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
     <cfRule type="duplicateValues" dxfId="18" priority="104"/>
@@ -29310,24 +30061,24 @@
     <cfRule type="duplicateValues" dxfId="16" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E401">
-    <cfRule type="duplicateValues" dxfId="15" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="8" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="7" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="4"/>
     <cfRule type="duplicateValues" dxfId="11" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="8" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E837:E840">
-    <cfRule type="duplicateValues" dxfId="7" priority="16" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="15" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="16" stopIfTrue="1"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A122" r:id="rId1" display="https://sellercentral.amazon.in/skucentral?mSku=FBA79849&amp;condition=New&amp;ref_=myp_skuc" xr:uid="{F5F7F880-2E3B-44E2-BABD-2E8055A5AAE6}"/>

</xml_diff>

<commit_message>
Week 18 data update: ads reports, inventory snapshots, processed datasets
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BAFB67-2ABB-4D1F-9E82-11318C988AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690AF3F8-13A2-4772-A982-B5FF5A7DE602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5121" uniqueCount="2817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5208" uniqueCount="2869">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -8488,6 +8488,162 @@
   </si>
   <si>
     <t>24 Channel Mixer With Carry Case</t>
+  </si>
+  <si>
+    <t>AA-26 Pro</t>
+  </si>
+  <si>
+    <t>FBA80124</t>
+  </si>
+  <si>
+    <t>AA-28</t>
+  </si>
+  <si>
+    <t>FBA80125</t>
+  </si>
+  <si>
+    <t>AA-29</t>
+  </si>
+  <si>
+    <t>FBA80126</t>
+  </si>
+  <si>
+    <t>AM-C49</t>
+  </si>
+  <si>
+    <t>B0GW8Z556N</t>
+  </si>
+  <si>
+    <t>FBA80009</t>
+  </si>
+  <si>
+    <t>FBA80010</t>
+  </si>
+  <si>
+    <t>FBA80119</t>
+  </si>
+  <si>
+    <t>FBA80120</t>
+  </si>
+  <si>
+    <t>AM-C50</t>
+  </si>
+  <si>
+    <t>AM-C51</t>
+  </si>
+  <si>
+    <t>AM-C52</t>
+  </si>
+  <si>
+    <t>AM-C53</t>
+  </si>
+  <si>
+    <t>AM-C54</t>
+  </si>
+  <si>
+    <t>SP-01</t>
+  </si>
+  <si>
+    <t>FBA79971</t>
+  </si>
+  <si>
+    <t>B0GGHZWMVW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nexlev </t>
+  </si>
+  <si>
+    <t>FBA79988</t>
+  </si>
+  <si>
+    <t>B0GN8N96R5</t>
+  </si>
+  <si>
+    <t>AP-04</t>
+  </si>
+  <si>
+    <t>FBA79989</t>
+  </si>
+  <si>
+    <t>B0GN86G345</t>
+  </si>
+  <si>
+    <t>CAP-05</t>
+  </si>
+  <si>
+    <t>FBA79992</t>
+  </si>
+  <si>
+    <t>B0GN94YDY2</t>
+  </si>
+  <si>
+    <t>ST-02</t>
+  </si>
+  <si>
+    <t>FBA79993</t>
+  </si>
+  <si>
+    <t>B0GN8WW6BC</t>
+  </si>
+  <si>
+    <t>ST-03</t>
+  </si>
+  <si>
+    <t>FBA80085</t>
+  </si>
+  <si>
+    <t>B0GXPBHDRF</t>
+  </si>
+  <si>
+    <t>M6</t>
+  </si>
+  <si>
+    <t>FBA80084</t>
+  </si>
+  <si>
+    <t>B0GXP97CZG</t>
+  </si>
+  <si>
+    <t>BE-4</t>
+  </si>
+  <si>
+    <t>FBA79984</t>
+  </si>
+  <si>
+    <t>B0GM1CZC7Y</t>
+  </si>
+  <si>
+    <t>MR-03</t>
+  </si>
+  <si>
+    <t>FBA80109</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t>FBA80110</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>FBA80121</t>
+  </si>
+  <si>
+    <t>AM-C55</t>
+  </si>
+  <si>
+    <t>FBA80122</t>
+  </si>
+  <si>
+    <t>AM-C56</t>
+  </si>
+  <si>
+    <t>FBA80123</t>
+  </si>
+  <si>
+    <t>AM-W25</t>
   </si>
 </sst>
 </file>
@@ -9355,13 +9511,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:I868"/>
+  <dimension ref="A1:I893"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.6640625" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.77734375" style="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.109375" style="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.88671875" style="13" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="50.88671875" style="13" bestFit="1" customWidth="1"/>
@@ -30010,6 +30166,332 @@
       </c>
       <c r="F868" s="13" t="s">
         <v>2661</v>
+      </c>
+    </row>
+    <row r="869" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A869" s="13" t="s">
+        <v>2818</v>
+      </c>
+      <c r="D869" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E869" s="13" t="s">
+        <v>2817</v>
+      </c>
+    </row>
+    <row r="870" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A870" s="13" t="s">
+        <v>2820</v>
+      </c>
+      <c r="D870" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E870" s="13" t="s">
+        <v>2819</v>
+      </c>
+    </row>
+    <row r="871" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A871" s="13" t="s">
+        <v>2822</v>
+      </c>
+      <c r="D871" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E871" s="13" t="s">
+        <v>2821</v>
+      </c>
+    </row>
+    <row r="872" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A872" s="13" t="s">
+        <v>720</v>
+      </c>
+      <c r="C872" s="13" t="s">
+        <v>2824</v>
+      </c>
+      <c r="D872" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E872" s="13" t="s">
+        <v>2823</v>
+      </c>
+    </row>
+    <row r="873" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A873" s="13" t="s">
+        <v>719</v>
+      </c>
+      <c r="D873" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E873" s="13" t="s">
+        <v>2829</v>
+      </c>
+    </row>
+    <row r="874" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A874" s="13" t="s">
+        <v>2825</v>
+      </c>
+      <c r="D874" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E874" s="13" t="s">
+        <v>2830</v>
+      </c>
+    </row>
+    <row r="875" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A875" s="13" t="s">
+        <v>2826</v>
+      </c>
+      <c r="D875" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E875" s="13" t="s">
+        <v>2831</v>
+      </c>
+    </row>
+    <row r="876" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A876" s="13" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D876" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E876" s="13" t="s">
+        <v>2832</v>
+      </c>
+    </row>
+    <row r="877" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A877" s="13" t="s">
+        <v>2828</v>
+      </c>
+      <c r="D877" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E877" s="13" t="s">
+        <v>2833</v>
+      </c>
+    </row>
+    <row r="878" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A878" s="13" t="s">
+        <v>2835</v>
+      </c>
+      <c r="C878" s="13" t="s">
+        <v>2836</v>
+      </c>
+      <c r="D878" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E878" s="13" t="s">
+        <v>2834</v>
+      </c>
+    </row>
+    <row r="879" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A879" s="13" t="s">
+        <v>2838</v>
+      </c>
+      <c r="C879" s="13" t="s">
+        <v>2839</v>
+      </c>
+      <c r="D879" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E879" s="13" t="s">
+        <v>2840</v>
+      </c>
+    </row>
+    <row r="880" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A880" s="13" t="s">
+        <v>2841</v>
+      </c>
+      <c r="C880" s="13" t="s">
+        <v>2842</v>
+      </c>
+      <c r="D880" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E880" s="13" t="s">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="881" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A881" s="13" t="s">
+        <v>2844</v>
+      </c>
+      <c r="C881" s="13" t="s">
+        <v>2845</v>
+      </c>
+      <c r="D881" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E881" s="13" t="s">
+        <v>2846</v>
+      </c>
+    </row>
+    <row r="882" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A882" s="13" t="s">
+        <v>2847</v>
+      </c>
+      <c r="C882" s="13" t="s">
+        <v>2848</v>
+      </c>
+      <c r="D882" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E882" s="13" t="s">
+        <v>2849</v>
+      </c>
+    </row>
+    <row r="883" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A883" s="13" t="s">
+        <v>2850</v>
+      </c>
+      <c r="C883" s="13" t="s">
+        <v>2851</v>
+      </c>
+      <c r="D883" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E883" s="13" t="s">
+        <v>2852</v>
+      </c>
+    </row>
+    <row r="884" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A884" s="13" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C884" s="13" t="s">
+        <v>2854</v>
+      </c>
+      <c r="D884" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E884" s="13" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="885" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A885" s="13" t="s">
+        <v>2856</v>
+      </c>
+      <c r="C885" s="13" t="s">
+        <v>2857</v>
+      </c>
+      <c r="D885" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E885" s="13" t="s">
+        <v>2858</v>
+      </c>
+    </row>
+    <row r="886" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A886" s="13" t="s">
+        <v>2841</v>
+      </c>
+      <c r="C886" s="13" t="s">
+        <v>2842</v>
+      </c>
+      <c r="D886" s="13" t="s">
+        <v>2837</v>
+      </c>
+      <c r="E886" s="13" t="s">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="887" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A887" s="13" t="s">
+        <v>2850</v>
+      </c>
+      <c r="C887" s="13" t="s">
+        <v>2851</v>
+      </c>
+      <c r="D887" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E887" s="13" t="s">
+        <v>2852</v>
+      </c>
+    </row>
+    <row r="888" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A888" s="13" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C888" s="13" t="s">
+        <v>2854</v>
+      </c>
+      <c r="D888" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E888" s="13" t="s">
+        <v>2855</v>
+      </c>
+    </row>
+    <row r="889" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A889" s="13" t="s">
+        <v>2859</v>
+      </c>
+      <c r="C889" s="13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D889" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E889" s="13" t="s">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="890" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A890" s="13" t="s">
+        <v>2861</v>
+      </c>
+      <c r="C890" s="13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D890" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E890" s="13" t="s">
+        <v>2862</v>
+      </c>
+    </row>
+    <row r="891" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A891" s="13" t="s">
+        <v>2863</v>
+      </c>
+      <c r="C891" s="13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D891" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E891" s="13" t="s">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="892" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A892" s="13" t="s">
+        <v>2865</v>
+      </c>
+      <c r="C892" s="13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D892" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E892" s="13" t="s">
+        <v>2866</v>
+      </c>
+    </row>
+    <row r="893" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A893" s="13" t="s">
+        <v>2867</v>
+      </c>
+      <c r="C893" s="13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D893" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E893" s="13" t="s">
+        <v>2868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: operator cleaned 21 raw exceptions + ETL refresh
Operator applied the action list from raw_exceptions_action_list.xlsx:

  • Added Tonor G11 ASINs to master (B0DTYHXMRQ, B0BVHZ5MKZ)
  • Filled 7 missing ASINs in Nexlev W10 B2B + W11 Pharmaeasy
  • Removed 5 'total' footer rows in Audio Array D2C sheets
  • Replaced 3 broken XLOOKUP formulas (Nexlev W15 ×2, WM W21 ×1)

Exceptions dropped: 27 → 6
Brand-populated rows in business_ads_joined: 1139 → 1141

Remaining (acceptable):
  • B0FR8XJFJ3 / B0GWPYFLWG / B0GWQ4T8MV — Audio Array W17 session-only
    listings, 0 sales (operator chose to ignore)
  • FBA79816 SKU-in-ASIN typo at W15 Audio_Array B2B row 25 (low impact,
    flagged for next cleanup)

Also adds scripts/generate_exception_action_list.py which produces a
per-row action sheet whenever the sync flags exceptions.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D66D190-EDCA-4956-8C2B-BD07590D461F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DEC919-39B7-4281-8051-60C91AC70208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6327" uniqueCount="3039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6332" uniqueCount="3041">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -9154,6 +9154,12 @@
   </si>
   <si>
     <t>B0GYS6CJD9</t>
+  </si>
+  <si>
+    <t>B0DTYHXMRQ</t>
+  </si>
+  <si>
+    <t>B0BVHZ5MKZ</t>
   </si>
 </sst>
 </file>
@@ -9375,20 +9381,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -9439,6 +9431,20 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -10041,7 +10047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:M917"/>
+  <dimension ref="A1:M918"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="13" bestFit="1" customWidth="1"/>
@@ -37629,6 +37635,9 @@
       <c r="A915" t="s">
         <v>3033</v>
       </c>
+      <c r="C915" s="13" t="s">
+        <v>3039</v>
+      </c>
       <c r="D915" s="13" t="s">
         <v>523</v>
       </c>
@@ -37662,6 +37671,20 @@
       </c>
       <c r="E917" s="13" t="s">
         <v>3036</v>
+      </c>
+    </row>
+    <row r="918" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A918" s="13" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C918" s="13" t="s">
+        <v>3040</v>
+      </c>
+      <c r="D918" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E918" s="13" t="s">
+        <v>1260</v>
       </c>
     </row>
   </sheetData>
@@ -37699,8 +37722,8 @@
     <cfRule type="duplicateValues" dxfId="21" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C98">
-    <cfRule type="duplicateValues" dxfId="20" priority="68"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E127:E143">
     <cfRule type="duplicateValues" dxfId="18" priority="63"/>
@@ -37720,13 +37743,13 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="E836:E839">
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="15" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
     <cfRule type="duplicateValues" dxfId="4" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="15" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="16" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:I1">
     <cfRule type="duplicateValues" dxfId="0" priority="107"/>

</xml_diff>

<commit_message>
chore(master): add bundle ASIN B0H2FCK54H (UB-06 = AM-S2 + AA-22)
Operator-added on 2026-05-28 to resolve the only ASIN_NOT_IN_MASTER
issue surfaced by the W21 inventory audit.  With this row in master,
the inventory ETL's ASIN-first alignment resolves cleanly for all
1,061 W21 inventory rows.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C6830BC-D0D3-4AA3-84B9-EE5C05804355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85C6266-F9AE-4AD6-AC76-677040D8152A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6332" uniqueCount="3041">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6333" uniqueCount="3042">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -9160,6 +9160,9 @@
   </si>
   <si>
     <t>B0BVHZ5MKZ</t>
+  </si>
+  <si>
+    <t>B0H2FCK54H</t>
   </si>
 </sst>
 </file>
@@ -9270,7 +9273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -9326,6 +9329,7 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -37147,7 +37151,9 @@
         <v>2869</v>
       </c>
       <c r="B898" s="5"/>
-      <c r="C898" s="5"/>
+      <c r="C898" s="19" t="s">
+        <v>3041</v>
+      </c>
       <c r="D898" s="5" t="s">
         <v>521</v>
       </c>

</xml_diff>

<commit_message>
tool(ads): LWA re-consent helper + W26 sku_master refresh
Adds scripts/ads_lwa_reconsent.py — self-contained OAuth flow for
regenerating AMS_ADS_REFRESH_TOKEN when the LWA consent expires or is
revoked.  Runs a local server on localhost:8765, catches the callback,
exchanges the code, enumerates profiles via /v2/profiles, and prints the
AdPilot-shape JSON blob ready to paste into the GitHub secret.

Also refreshes data/master/sku_master.xlsx per operator update.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78574D12-5D4A-40AE-9E54-B7328B11C4AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71EEFFE6-1D31-4ED3-98A8-D814A544D0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$3007</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$3009</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16769" uniqueCount="9295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16781" uniqueCount="9298">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -27922,6 +27922,15 @@
   </si>
   <si>
     <t>B0FTKJC5JW</t>
+  </si>
+  <si>
+    <t>FBA80181</t>
+  </si>
+  <si>
+    <t>AI-04 Pro</t>
+  </si>
+  <si>
+    <t>B0H2FNV2RC</t>
   </si>
 </sst>
 </file>
@@ -28783,7 +28792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:M3007"/>
+  <dimension ref="A1:M3009"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -91716,7 +91725,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2993" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2993" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2993" s="2" t="s">
         <v>7203</v>
       </c>
@@ -91733,7 +91742,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2994" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2994" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2994" s="2" t="s">
         <v>7204</v>
       </c>
@@ -91750,7 +91759,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2995" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2995" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2995" s="2" t="s">
         <v>7205</v>
       </c>
@@ -91767,7 +91776,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2996" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2996" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2996" s="2" t="s">
         <v>7206</v>
       </c>
@@ -91784,7 +91793,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2997" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2997" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2997" s="2" t="s">
         <v>7207</v>
       </c>
@@ -91801,7 +91810,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2998" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2998" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2998" s="2">
         <v>0</v>
       </c>
@@ -91818,7 +91827,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="2999" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2999" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2999" s="2">
         <v>0</v>
       </c>
@@ -91835,7 +91844,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3000" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3000" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3000" s="2" t="s">
         <v>7208</v>
       </c>
@@ -91852,7 +91861,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3001" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3001" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3001" s="2" t="s">
         <v>7209</v>
       </c>
@@ -91869,7 +91878,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3002" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3002" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3002" s="2" t="s">
         <v>7210</v>
       </c>
@@ -91886,7 +91895,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3003" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3003" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3003" s="2" t="s">
         <v>7211</v>
       </c>
@@ -91903,7 +91912,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3004" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3004" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3004" s="2" t="s">
         <v>7212</v>
       </c>
@@ -91920,7 +91929,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3005" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3005" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3005" s="2" t="s">
         <v>7213</v>
       </c>
@@ -91937,7 +91946,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3006" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3006" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3006" s="2" t="s">
         <v>7214</v>
       </c>
@@ -91954,7 +91963,7 @@
         <v>2645</v>
       </c>
     </row>
-    <row r="3007" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3007" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3007" s="2" t="s">
         <v>7215</v>
       </c>
@@ -91969,6 +91978,46 @@
       </c>
       <c r="J3007" s="5" t="s">
         <v>2645</v>
+      </c>
+    </row>
+    <row r="3008" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3008" s="2" t="s">
+        <v>9295</v>
+      </c>
+      <c r="D3008" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="E3008" s="2" t="s">
+        <v>9296</v>
+      </c>
+      <c r="G3008" s="2" t="s">
+        <v>2954</v>
+      </c>
+      <c r="J3008" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="K3008" s="2" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="3009" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3009" s="2" t="s">
+        <v>2868</v>
+      </c>
+      <c r="C3009" s="2" t="s">
+        <v>9297</v>
+      </c>
+      <c r="D3009" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="E3009" s="2" t="s">
+        <v>2896</v>
+      </c>
+      <c r="J3009" s="2" t="s">
+        <v>1125</v>
+      </c>
+      <c r="K3009" s="2" t="s">
+        <v>2917</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(W35): Flipkart late-landing re-pull + 33 new Fossil ASINs in sku_master
- oms_other_channels --week 35 re-pull: Flipkart Rs11,198 (AA, 2 asins/4u)
  landed in OMS after the original Monday pull; D2C-AA +Rs2,013 drift.
  W35 total now Rs1,22,48,169. Fossil/Amazon/1P untouched to the rupee.
- sku_master: +33 Fossil rows (pure fill verified cell-by-cell — zero
  existing rows changed). All 33 are unlaunched (zero sales W28-35);
  mapping is forward-looking for when they go live.
- sanity gate OK (823 rows/3,607u vs floor 820/3,602); audit's '33 absent
  from downstream' = exactly these unlaunched Fossil ASINs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nner8RaGyk95YsJkMTo8Tg
</commit_message>
<xml_diff>
--- a/data/master/sku_master.xlsx
+++ b/data/master/sku_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E66BC89-0C0A-45A7-9C57-06BC79507239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93541365-ACED-4337-978C-5E9A4F9468AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{117C6BDF-C413-4A9B-8C98-0B7CEC880D6C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17439" uniqueCount="9404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17604" uniqueCount="9503">
   <si>
     <t>FBA SKU</t>
   </si>
@@ -28252,6 +28252,303 @@
   </si>
   <si>
     <t>T-Code (EAN)</t>
+  </si>
+  <si>
+    <t>B07WGWGMBM</t>
+  </si>
+  <si>
+    <t>B0H1K1XJBK</t>
+  </si>
+  <si>
+    <t>B0H1JTMVMW</t>
+  </si>
+  <si>
+    <t>B0H1K4MHH4</t>
+  </si>
+  <si>
+    <t>B0H1JZFQRZ</t>
+  </si>
+  <si>
+    <t>B0H1K1W6GJ</t>
+  </si>
+  <si>
+    <t>B0H44QP75W</t>
+  </si>
+  <si>
+    <t>B0H44XPFRC</t>
+  </si>
+  <si>
+    <t>B0H8XG2F43</t>
+  </si>
+  <si>
+    <t>B0H8XXYKBC</t>
+  </si>
+  <si>
+    <t>B0H8Y4Z1KK</t>
+  </si>
+  <si>
+    <t>B0H1K56S6V</t>
+  </si>
+  <si>
+    <t>B0H1K216VW</t>
+  </si>
+  <si>
+    <t>B0H1JTL93N</t>
+  </si>
+  <si>
+    <t>B0H8Y38KKY</t>
+  </si>
+  <si>
+    <t>B0H1K2HBC9</t>
+  </si>
+  <si>
+    <t>B0H1KB3F39</t>
+  </si>
+  <si>
+    <t>B0H1K5RK6V</t>
+  </si>
+  <si>
+    <t>B0H8XZ9N1P</t>
+  </si>
+  <si>
+    <t>B0H1K4MHGJ</t>
+  </si>
+  <si>
+    <t>B0H1JY5HK3</t>
+  </si>
+  <si>
+    <t>B0H1JN7L2Z</t>
+  </si>
+  <si>
+    <t>B0H2ZX1W6F</t>
+  </si>
+  <si>
+    <t>B0H2ZVD5RS</t>
+  </si>
+  <si>
+    <t>B0H312FS95</t>
+  </si>
+  <si>
+    <t>B0H2ZX6LSV</t>
+  </si>
+  <si>
+    <t>B0H2ZMP3LX</t>
+  </si>
+  <si>
+    <t>B0H2ZZQDC9</t>
+  </si>
+  <si>
+    <t>B0H2ZPG58N</t>
+  </si>
+  <si>
+    <t>B0H1JXJ5LV</t>
+  </si>
+  <si>
+    <t>B0H1K1N4X4</t>
+  </si>
+  <si>
+    <t>B0H2ZT21NJ</t>
+  </si>
+  <si>
+    <t>B0H2ZR4K77</t>
+  </si>
+  <si>
+    <t>FBA80118</t>
+  </si>
+  <si>
+    <t>FBA80257</t>
+  </si>
+  <si>
+    <t>FBA80258</t>
+  </si>
+  <si>
+    <t>FBA80259</t>
+  </si>
+  <si>
+    <t>FBA80262</t>
+  </si>
+  <si>
+    <t>FBA80263</t>
+  </si>
+  <si>
+    <t>FBA80265</t>
+  </si>
+  <si>
+    <t>FBA80266</t>
+  </si>
+  <si>
+    <t>FBA80268</t>
+  </si>
+  <si>
+    <t>FBA80269</t>
+  </si>
+  <si>
+    <t>FBA80270</t>
+  </si>
+  <si>
+    <t>FBA80271</t>
+  </si>
+  <si>
+    <t>FBA80272</t>
+  </si>
+  <si>
+    <t>FBA80273</t>
+  </si>
+  <si>
+    <t>FBA80274</t>
+  </si>
+  <si>
+    <t>FBA80275</t>
+  </si>
+  <si>
+    <t>FBA80276</t>
+  </si>
+  <si>
+    <t>FBA80277</t>
+  </si>
+  <si>
+    <t>FBA80278</t>
+  </si>
+  <si>
+    <t>FBA80279</t>
+  </si>
+  <si>
+    <t>FBA80280</t>
+  </si>
+  <si>
+    <t>FBA80281</t>
+  </si>
+  <si>
+    <t>FBA80282</t>
+  </si>
+  <si>
+    <t>FBA80283</t>
+  </si>
+  <si>
+    <t>FBA80284</t>
+  </si>
+  <si>
+    <t>FBA80285</t>
+  </si>
+  <si>
+    <t>FBA80288</t>
+  </si>
+  <si>
+    <t>FBA80290</t>
+  </si>
+  <si>
+    <t>FBA80292</t>
+  </si>
+  <si>
+    <t>FBA80260</t>
+  </si>
+  <si>
+    <t>FBA80261</t>
+  </si>
+  <si>
+    <t>FBA80286</t>
+  </si>
+  <si>
+    <t>FBA80289</t>
+  </si>
+  <si>
+    <t>FS5661</t>
+  </si>
+  <si>
+    <t>AX2467</t>
+  </si>
+  <si>
+    <t>AX2468</t>
+  </si>
+  <si>
+    <t>AX2652</t>
+  </si>
+  <si>
+    <t>AX4409</t>
+  </si>
+  <si>
+    <t>AX4410</t>
+  </si>
+  <si>
+    <t>DZ4715</t>
+  </si>
+  <si>
+    <t>DZ4724</t>
+  </si>
+  <si>
+    <t>CE1135</t>
+  </si>
+  <si>
+    <t>CE1136</t>
+  </si>
+  <si>
+    <t>CE1137</t>
+  </si>
+  <si>
+    <t>ES5503</t>
+  </si>
+  <si>
+    <t>ES5504</t>
+  </si>
+  <si>
+    <t>ES5505</t>
+  </si>
+  <si>
+    <t>ES5512</t>
+  </si>
+  <si>
+    <t>FS6180</t>
+  </si>
+  <si>
+    <t>FS6181</t>
+  </si>
+  <si>
+    <t>FS6182</t>
+  </si>
+  <si>
+    <t>FS6189</t>
+  </si>
+  <si>
+    <t>FS6194</t>
+  </si>
+  <si>
+    <t>FS6198SET</t>
+  </si>
+  <si>
+    <t>FS6199SET</t>
+  </si>
+  <si>
+    <t>MK7618</t>
+  </si>
+  <si>
+    <t>MK7619</t>
+  </si>
+  <si>
+    <t>MK7620</t>
+  </si>
+  <si>
+    <t>MK7621</t>
+  </si>
+  <si>
+    <t>MK7641</t>
+  </si>
+  <si>
+    <t>MK9273</t>
+  </si>
+  <si>
+    <t>MK9277</t>
+  </si>
+  <si>
+    <t>AX4174</t>
+  </si>
+  <si>
+    <t>AX4175</t>
+  </si>
+  <si>
+    <t>MK7626</t>
+  </si>
+  <si>
+    <t>MK7642</t>
   </si>
 </sst>
 </file>
@@ -28474,28 +28771,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -28558,6 +28833,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -28570,6 +28865,8 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -29584,7 +29881,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B2CFDDD-D63B-4FDB-9746-BFEFFD00084B}">
-  <dimension ref="A1:S3041"/>
+  <dimension ref="A1:S3074"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" style="2" bestFit="1" customWidth="1"/>
@@ -95491,6 +95788,567 @@
       </c>
       <c r="P3041" s="2" t="e">
         <v>#N/A</v>
+      </c>
+    </row>
+    <row r="3042" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3042" s="2" t="s">
+        <v>9437</v>
+      </c>
+      <c r="C3042" s="2" t="s">
+        <v>9404</v>
+      </c>
+      <c r="D3042" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3042" s="2" t="s">
+        <v>9470</v>
+      </c>
+      <c r="J3042" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3043" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3043" s="2" t="s">
+        <v>9438</v>
+      </c>
+      <c r="C3043" s="2" t="s">
+        <v>9405</v>
+      </c>
+      <c r="D3043" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3043" s="2" t="s">
+        <v>9471</v>
+      </c>
+      <c r="J3043" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3044" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3044" s="2" t="s">
+        <v>9439</v>
+      </c>
+      <c r="C3044" s="2" t="s">
+        <v>9406</v>
+      </c>
+      <c r="D3044" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3044" s="2" t="s">
+        <v>9472</v>
+      </c>
+      <c r="J3044" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3045" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3045" s="2" t="s">
+        <v>9440</v>
+      </c>
+      <c r="C3045" s="2" t="s">
+        <v>9407</v>
+      </c>
+      <c r="D3045" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3045" s="2" t="s">
+        <v>9473</v>
+      </c>
+      <c r="J3045" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3046" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3046" s="2" t="s">
+        <v>9441</v>
+      </c>
+      <c r="C3046" s="2" t="s">
+        <v>9408</v>
+      </c>
+      <c r="D3046" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3046" s="2" t="s">
+        <v>9474</v>
+      </c>
+      <c r="J3046" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3047" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3047" s="2" t="s">
+        <v>9442</v>
+      </c>
+      <c r="C3047" s="2" t="s">
+        <v>9409</v>
+      </c>
+      <c r="D3047" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3047" s="2" t="s">
+        <v>9475</v>
+      </c>
+      <c r="J3047" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3048" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3048" s="2" t="s">
+        <v>9443</v>
+      </c>
+      <c r="C3048" s="2" t="s">
+        <v>9410</v>
+      </c>
+      <c r="D3048" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3048" s="2" t="s">
+        <v>9476</v>
+      </c>
+      <c r="J3048" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3049" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3049" s="2" t="s">
+        <v>9444</v>
+      </c>
+      <c r="C3049" s="2" t="s">
+        <v>9411</v>
+      </c>
+      <c r="D3049" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3049" s="2" t="s">
+        <v>9477</v>
+      </c>
+      <c r="J3049" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3050" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3050" s="2" t="s">
+        <v>9445</v>
+      </c>
+      <c r="C3050" s="2" t="s">
+        <v>9412</v>
+      </c>
+      <c r="D3050" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3050" s="2" t="s">
+        <v>9478</v>
+      </c>
+      <c r="J3050" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3051" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3051" s="2" t="s">
+        <v>9446</v>
+      </c>
+      <c r="C3051" s="2" t="s">
+        <v>9413</v>
+      </c>
+      <c r="D3051" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3051" s="2" t="s">
+        <v>9479</v>
+      </c>
+      <c r="J3051" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3052" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3052" s="2" t="s">
+        <v>9447</v>
+      </c>
+      <c r="C3052" s="2" t="s">
+        <v>9414</v>
+      </c>
+      <c r="D3052" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3052" s="2" t="s">
+        <v>9480</v>
+      </c>
+      <c r="J3052" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3053" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3053" s="2" t="s">
+        <v>9448</v>
+      </c>
+      <c r="C3053" s="2" t="s">
+        <v>9415</v>
+      </c>
+      <c r="D3053" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3053" s="2" t="s">
+        <v>9481</v>
+      </c>
+      <c r="J3053" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3054" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3054" s="2" t="s">
+        <v>9449</v>
+      </c>
+      <c r="C3054" s="2" t="s">
+        <v>9416</v>
+      </c>
+      <c r="D3054" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3054" s="2" t="s">
+        <v>9482</v>
+      </c>
+      <c r="J3054" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3055" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3055" s="2" t="s">
+        <v>9450</v>
+      </c>
+      <c r="C3055" s="2" t="s">
+        <v>9417</v>
+      </c>
+      <c r="D3055" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3055" s="2" t="s">
+        <v>9483</v>
+      </c>
+      <c r="J3055" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3056" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3056" s="2" t="s">
+        <v>9451</v>
+      </c>
+      <c r="C3056" s="2" t="s">
+        <v>9418</v>
+      </c>
+      <c r="D3056" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3056" s="2" t="s">
+        <v>9484</v>
+      </c>
+      <c r="J3056" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3057" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3057" s="2" t="s">
+        <v>9452</v>
+      </c>
+      <c r="C3057" s="2" t="s">
+        <v>9419</v>
+      </c>
+      <c r="D3057" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3057" s="2" t="s">
+        <v>9485</v>
+      </c>
+      <c r="J3057" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3058" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3058" s="2" t="s">
+        <v>9453</v>
+      </c>
+      <c r="C3058" s="2" t="s">
+        <v>9420</v>
+      </c>
+      <c r="D3058" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3058" s="2" t="s">
+        <v>9486</v>
+      </c>
+      <c r="J3058" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3059" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3059" s="2" t="s">
+        <v>9454</v>
+      </c>
+      <c r="C3059" s="2" t="s">
+        <v>9421</v>
+      </c>
+      <c r="D3059" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3059" s="2" t="s">
+        <v>9487</v>
+      </c>
+      <c r="J3059" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3060" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3060" s="2" t="s">
+        <v>9455</v>
+      </c>
+      <c r="C3060" s="2" t="s">
+        <v>9422</v>
+      </c>
+      <c r="D3060" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3060" s="2" t="s">
+        <v>9488</v>
+      </c>
+      <c r="J3060" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3061" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3061" s="2" t="s">
+        <v>9456</v>
+      </c>
+      <c r="C3061" s="2" t="s">
+        <v>9423</v>
+      </c>
+      <c r="D3061" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3061" s="2" t="s">
+        <v>9489</v>
+      </c>
+      <c r="J3061" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3062" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3062" s="2" t="s">
+        <v>9457</v>
+      </c>
+      <c r="C3062" s="2" t="s">
+        <v>9424</v>
+      </c>
+      <c r="D3062" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3062" s="2" t="s">
+        <v>9490</v>
+      </c>
+      <c r="J3062" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3063" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3063" s="2" t="s">
+        <v>9458</v>
+      </c>
+      <c r="C3063" s="2" t="s">
+        <v>9425</v>
+      </c>
+      <c r="D3063" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3063" s="2" t="s">
+        <v>9491</v>
+      </c>
+      <c r="J3063" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3064" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3064" s="2" t="s">
+        <v>9459</v>
+      </c>
+      <c r="C3064" s="2" t="s">
+        <v>9426</v>
+      </c>
+      <c r="D3064" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3064" s="2" t="s">
+        <v>9492</v>
+      </c>
+      <c r="J3064" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3065" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3065" s="2" t="s">
+        <v>9460</v>
+      </c>
+      <c r="C3065" s="2" t="s">
+        <v>9427</v>
+      </c>
+      <c r="D3065" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3065" s="2" t="s">
+        <v>9493</v>
+      </c>
+      <c r="J3065" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3066" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3066" s="2" t="s">
+        <v>9461</v>
+      </c>
+      <c r="C3066" s="2" t="s">
+        <v>9428</v>
+      </c>
+      <c r="D3066" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3066" s="2" t="s">
+        <v>9494</v>
+      </c>
+      <c r="J3066" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3067" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3067" s="2" t="s">
+        <v>9462</v>
+      </c>
+      <c r="C3067" s="2" t="s">
+        <v>9429</v>
+      </c>
+      <c r="D3067" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3067" s="2" t="s">
+        <v>9495</v>
+      </c>
+      <c r="J3067" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3068" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3068" s="2" t="s">
+        <v>9463</v>
+      </c>
+      <c r="C3068" s="2" t="s">
+        <v>9430</v>
+      </c>
+      <c r="D3068" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3068" s="2" t="s">
+        <v>9496</v>
+      </c>
+      <c r="J3068" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3069" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3069" s="2" t="s">
+        <v>9464</v>
+      </c>
+      <c r="C3069" s="2" t="s">
+        <v>9431</v>
+      </c>
+      <c r="D3069" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3069" s="2" t="s">
+        <v>9497</v>
+      </c>
+      <c r="J3069" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3070" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3070" s="2" t="s">
+        <v>9465</v>
+      </c>
+      <c r="C3070" s="2" t="s">
+        <v>9432</v>
+      </c>
+      <c r="D3070" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3070" s="2" t="s">
+        <v>9498</v>
+      </c>
+      <c r="J3070" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3071" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3071" s="2" t="s">
+        <v>9466</v>
+      </c>
+      <c r="C3071" s="2" t="s">
+        <v>9433</v>
+      </c>
+      <c r="D3071" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3071" s="2" t="s">
+        <v>9499</v>
+      </c>
+      <c r="J3071" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3072" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3072" s="2" t="s">
+        <v>9467</v>
+      </c>
+      <c r="C3072" s="2" t="s">
+        <v>9434</v>
+      </c>
+      <c r="D3072" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3072" s="2" t="s">
+        <v>9500</v>
+      </c>
+      <c r="J3072" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3073" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3073" s="2" t="s">
+        <v>9468</v>
+      </c>
+      <c r="C3073" s="2" t="s">
+        <v>9435</v>
+      </c>
+      <c r="D3073" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3073" s="2" t="s">
+        <v>9501</v>
+      </c>
+      <c r="J3073" s="2" t="s">
+        <v>2644</v>
+      </c>
+    </row>
+    <row r="3074" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3074" s="2" t="s">
+        <v>9469</v>
+      </c>
+      <c r="C3074" s="2" t="s">
+        <v>9436</v>
+      </c>
+      <c r="D3074" s="2" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E3074" s="2" t="s">
+        <v>9502</v>
+      </c>
+      <c r="J3074" s="2" t="s">
+        <v>2644</v>
       </c>
     </row>
   </sheetData>
@@ -95518,8 +96376,8 @@
     <cfRule type="duplicateValues" dxfId="34" priority="101"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="duplicateValues" dxfId="33" priority="81"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B125">
     <cfRule type="duplicateValues" dxfId="31" priority="78"/>
@@ -95539,9 +96397,9 @@
     <cfRule type="duplicateValues" dxfId="25" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E400">
-    <cfRule type="duplicateValues" dxfId="24" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="10"/>
     <cfRule type="duplicateValues" dxfId="21" priority="12"/>
     <cfRule type="duplicateValues" dxfId="20" priority="13"/>
     <cfRule type="duplicateValues" dxfId="19" priority="14"/>
@@ -95549,23 +96407,23 @@
     <cfRule type="duplicateValues" dxfId="17" priority="16" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E837:E840">
-    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
-    <cfRule type="duplicateValues" dxfId="15" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="21"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="23" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="23" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="24" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3010">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="7" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
     <cfRule type="duplicateValues" dxfId="1" priority="8" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:I1">

</xml_diff>